<commit_message>
solo faltan 9 carnets!
</commit_message>
<xml_diff>
--- a/Datos Tesis Upstream/Algoritmos y Programacion/2425-2/Partic.Alg 2425-2 Secc. 1.xlsx
+++ b/Datos Tesis Upstream/Algoritmos y Programacion/2425-2/Partic.Alg 2425-2 Secc. 1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nelsoncarrillo/Downloads/tesis-prediccion-participacion/Datos Tesis Upstream/Algoritmos y Programacion/2425-2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{556CA100-DA41-9D48-990E-727010EAF521}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F28C20C0-33E8-174B-9803-E05BE73E6AC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15980" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,6 @@
     <sheet name="Estandar" sheetId="11" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -59,6 +58,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Recuperación Sem 12
@@ -83,6 +83,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>======
@@ -99,6 +100,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>partic. alta
@@ -113,6 +115,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>======
@@ -129,6 +132,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -143,6 +147,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -157,6 +162,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>======
@@ -173,6 +179,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>======
@@ -189,6 +196,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>======
@@ -205,6 +213,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -219,6 +228,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -233,6 +243,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -247,6 +258,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -261,6 +273,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Dinámica
@@ -275,6 +288,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>======
@@ -291,6 +305,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>======
@@ -307,6 +322,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>======
@@ -323,6 +339,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -337,6 +354,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -351,6 +369,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -365,6 +384,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -379,6 +399,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -394,6 +415,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea y Dinámica
@@ -408,6 +430,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -422,6 +445,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>======
@@ -438,6 +462,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -452,6 +477,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -466,6 +492,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -480,6 +507,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -494,6 +522,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -508,6 +537,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>======
@@ -524,6 +554,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>======
@@ -540,6 +571,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -554,6 +586,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -569,6 +602,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Dinámica
@@ -583,6 +617,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -597,6 +632,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -611,6 +647,7 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -634,13 +671,14 @@
     <author/>
   </authors>
   <commentList>
-    <comment ref="G9" authorId="0" shapeId="0" xr:uid="{994E8CB0-49CB-3545-87B6-2362AAFCA677}">
+    <comment ref="H9" authorId="0" shapeId="0" xr:uid="{994E8CB0-49CB-3545-87B6-2362AAFCA677}">
       <text>
         <r>
           <rPr>
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>======
@@ -650,13 +688,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="P9" authorId="0" shapeId="0" xr:uid="{62B7A32A-8C0D-304B-B21A-85FC14FE7167}">
+    <comment ref="Q9" authorId="0" shapeId="0" xr:uid="{62B7A32A-8C0D-304B-B21A-85FC14FE7167}">
       <text>
         <r>
           <rPr>
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -664,13 +703,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="S9" authorId="0" shapeId="0" xr:uid="{6548CB0E-96B2-6948-8788-20433F669065}">
+    <comment ref="T9" authorId="0" shapeId="0" xr:uid="{6548CB0E-96B2-6948-8788-20433F669065}">
       <text>
         <r>
           <rPr>
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -678,13 +718,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="G11" authorId="0" shapeId="0" xr:uid="{0468BF06-317B-3746-AEA4-F90B0E05FC8E}">
+    <comment ref="H11" authorId="0" shapeId="0" xr:uid="{0468BF06-317B-3746-AEA4-F90B0E05FC8E}">
       <text>
         <r>
           <rPr>
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>======
@@ -694,13 +735,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="I15" authorId="0" shapeId="0" xr:uid="{A25B3EAB-6DF5-5E4C-B61E-94E268A78F85}">
+    <comment ref="J15" authorId="0" shapeId="0" xr:uid="{A25B3EAB-6DF5-5E4C-B61E-94E268A78F85}">
       <text>
         <r>
           <rPr>
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -708,13 +750,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="K15" authorId="0" shapeId="0" xr:uid="{9D76DEF9-E673-4D4E-B25E-CFB77F55766D}">
+    <comment ref="L15" authorId="0" shapeId="0" xr:uid="{9D76DEF9-E673-4D4E-B25E-CFB77F55766D}">
       <text>
         <r>
           <rPr>
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -722,13 +765,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="S15" authorId="0" shapeId="0" xr:uid="{71E32D29-685E-5945-BBF3-1FA464FDE009}">
+    <comment ref="T15" authorId="0" shapeId="0" xr:uid="{71E32D29-685E-5945-BBF3-1FA464FDE009}">
       <text>
         <r>
           <rPr>
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -736,13 +780,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="I16" authorId="0" shapeId="0" xr:uid="{BF91A6AB-E26F-884D-8C2F-235117C30B59}">
+    <comment ref="J16" authorId="0" shapeId="0" xr:uid="{BF91A6AB-E26F-884D-8C2F-235117C30B59}">
       <text>
         <r>
           <rPr>
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -750,13 +795,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="P16" authorId="0" shapeId="0" xr:uid="{9FAC2580-2975-4E45-B18C-1E5E7F8ABB53}">
+    <comment ref="Q16" authorId="0" shapeId="0" xr:uid="{9FAC2580-2975-4E45-B18C-1E5E7F8ABB53}">
       <text>
         <r>
           <rPr>
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Dinámica
@@ -764,29 +810,57 @@
         </r>
       </text>
     </comment>
-    <comment ref="G17" authorId="0" shapeId="0" xr:uid="{2D7A3FD8-AE8B-7D43-B03F-C94FD0FD7518}">
+    <comment ref="H17" authorId="0" shapeId="0" xr:uid="{2D7A3FD8-AE8B-7D43-B03F-C94FD0FD7518}">
       <text>
         <r>
           <rPr>
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
-            <scheme val="minor"/>
+            <family val="2"/>
           </rPr>
-          <t>======
-ID#AAABbmVhGZo
-Fernando Torre    (2025-01-13 20:58:36)
-Tarea 1/2</t>
+          <t xml:space="preserve">======
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">ID#AAABbmVhGZo
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Fernando Torre    (2025-01-13 20:58:36)
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>Tarea 1/2</t>
         </r>
       </text>
     </comment>
-    <comment ref="G20" authorId="0" shapeId="0" xr:uid="{CC76BF2A-E6A1-9745-801E-C4656E9ABF9C}">
+    <comment ref="H20" authorId="0" shapeId="0" xr:uid="{CC76BF2A-E6A1-9745-801E-C4656E9ABF9C}">
       <text>
         <r>
           <rPr>
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>======
@@ -796,13 +870,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="H20" authorId="0" shapeId="0" xr:uid="{AC1290A2-09DB-4B4B-96AE-2D8300577FD3}">
+    <comment ref="I20" authorId="0" shapeId="0" xr:uid="{AC1290A2-09DB-4B4B-96AE-2D8300577FD3}">
       <text>
         <r>
           <rPr>
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -810,13 +885,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="K21" authorId="0" shapeId="0" xr:uid="{FE5D04D3-30C8-5248-A9F8-01F10D91DC19}">
+    <comment ref="L21" authorId="0" shapeId="0" xr:uid="{FE5D04D3-30C8-5248-A9F8-01F10D91DC19}">
       <text>
         <r>
           <rPr>
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -824,13 +900,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q21" authorId="0" shapeId="0" xr:uid="{9AB704A9-0D4A-DD43-B2C5-FC6814A6E63F}">
+    <comment ref="R21" authorId="0" shapeId="0" xr:uid="{9AB704A9-0D4A-DD43-B2C5-FC6814A6E63F}">
       <text>
         <r>
           <rPr>
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -838,13 +915,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="I24" authorId="0" shapeId="0" xr:uid="{4EA10B4B-2772-7041-BE80-0D81EC79DD4D}">
+    <comment ref="J24" authorId="0" shapeId="0" xr:uid="{4EA10B4B-2772-7041-BE80-0D81EC79DD4D}">
       <text>
         <r>
           <rPr>
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -852,13 +930,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="J24" authorId="0" shapeId="0" xr:uid="{9188C0EA-B879-5A4D-B6EA-E1DC7B6D0155}">
+    <comment ref="K24" authorId="0" shapeId="0" xr:uid="{9188C0EA-B879-5A4D-B6EA-E1DC7B6D0155}">
       <text>
         <r>
           <rPr>
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -867,13 +946,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="P24" authorId="0" shapeId="0" xr:uid="{204D0ECE-1FAB-D343-B51E-F6A1C37895AE}">
+    <comment ref="Q24" authorId="0" shapeId="0" xr:uid="{204D0ECE-1FAB-D343-B51E-F6A1C37895AE}">
       <text>
         <r>
           <rPr>
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea y Dinámica
@@ -881,13 +961,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="R24" authorId="0" shapeId="0" xr:uid="{363A62D1-EB87-5C40-9A77-0E9E7B83AED7}">
+    <comment ref="S24" authorId="0" shapeId="0" xr:uid="{363A62D1-EB87-5C40-9A77-0E9E7B83AED7}">
       <text>
         <r>
           <rPr>
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -895,13 +976,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="G26" authorId="0" shapeId="0" xr:uid="{A05E896E-AEB5-6449-A9A0-5CD4E823C28B}">
+    <comment ref="H26" authorId="0" shapeId="0" xr:uid="{A05E896E-AEB5-6449-A9A0-5CD4E823C28B}">
       <text>
         <r>
           <rPr>
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>======
@@ -911,13 +993,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="P28" authorId="0" shapeId="0" xr:uid="{AD378E21-BA7A-6141-A939-1386B810BBF0}">
+    <comment ref="Q28" authorId="0" shapeId="0" xr:uid="{AD378E21-BA7A-6141-A939-1386B810BBF0}">
       <text>
         <r>
           <rPr>
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -925,13 +1008,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q28" authorId="0" shapeId="0" xr:uid="{5D6DB1A7-E969-AD49-950F-8706A5CE779E}">
+    <comment ref="R28" authorId="0" shapeId="0" xr:uid="{5D6DB1A7-E969-AD49-950F-8706A5CE779E}">
       <text>
         <r>
           <rPr>
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -939,13 +1023,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="R28" authorId="0" shapeId="0" xr:uid="{C95B9813-A03A-174F-B026-14C5755DDDB0}">
+    <comment ref="S28" authorId="0" shapeId="0" xr:uid="{C95B9813-A03A-174F-B026-14C5755DDDB0}">
       <text>
         <r>
           <rPr>
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -953,13 +1038,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="H29" authorId="0" shapeId="0" xr:uid="{069DC1D5-A2EF-D043-9197-68F1DBA36891}">
+    <comment ref="I29" authorId="0" shapeId="0" xr:uid="{069DC1D5-A2EF-D043-9197-68F1DBA36891}">
       <text>
         <r>
           <rPr>
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -967,13 +1053,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="H33" authorId="0" shapeId="0" xr:uid="{A290E633-4242-FF45-B601-5B400A42C14F}">
+    <comment ref="I33" authorId="0" shapeId="0" xr:uid="{A290E633-4242-FF45-B601-5B400A42C14F}">
       <text>
         <r>
           <rPr>
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -981,13 +1068,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="G34" authorId="0" shapeId="0" xr:uid="{AA80A1BA-195C-2149-A5CF-2003FEAE0BD0}">
+    <comment ref="H34" authorId="0" shapeId="0" xr:uid="{AA80A1BA-195C-2149-A5CF-2003FEAE0BD0}">
       <text>
         <r>
           <rPr>
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>======
@@ -997,13 +1085,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="H34" authorId="0" shapeId="0" xr:uid="{4DB83B3C-CD28-D349-A796-AFC0781C7DC1}">
+    <comment ref="I34" authorId="0" shapeId="0" xr:uid="{4DB83B3C-CD28-D349-A796-AFC0781C7DC1}">
       <text>
         <r>
           <rPr>
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -1011,13 +1100,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="J34" authorId="0" shapeId="0" xr:uid="{EB636BF7-F8C5-364E-8DFF-CE8441657C32}">
+    <comment ref="K34" authorId="0" shapeId="0" xr:uid="{EB636BF7-F8C5-364E-8DFF-CE8441657C32}">
       <text>
         <r>
           <rPr>
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -1026,13 +1116,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q34" authorId="0" shapeId="0" xr:uid="{028FEE78-C371-6647-AEBC-E2C54F102C5B}">
+    <comment ref="R34" authorId="0" shapeId="0" xr:uid="{028FEE78-C371-6647-AEBC-E2C54F102C5B}">
       <text>
         <r>
           <rPr>
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Dinámica
@@ -1040,13 +1131,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="H36" authorId="0" shapeId="0" xr:uid="{54E4D6B4-C125-A747-8C66-48345C6F928D}">
+    <comment ref="I36" authorId="0" shapeId="0" xr:uid="{54E4D6B4-C125-A747-8C66-48345C6F928D}">
       <text>
         <r>
           <rPr>
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -1054,13 +1146,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="I36" authorId="0" shapeId="0" xr:uid="{B7E2D48F-7052-7248-ABB2-9C21566265B7}">
+    <comment ref="J36" authorId="0" shapeId="0" xr:uid="{B7E2D48F-7052-7248-ABB2-9C21566265B7}">
       <text>
         <r>
           <rPr>
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -1068,13 +1161,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="J36" authorId="0" shapeId="0" xr:uid="{F96959EB-8E3E-FE44-8A18-D7DCED7104C4}">
+    <comment ref="K36" authorId="0" shapeId="0" xr:uid="{F96959EB-8E3E-FE44-8A18-D7DCED7104C4}">
       <text>
         <r>
           <rPr>
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Tarea
@@ -1088,7 +1182,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="978" uniqueCount="531">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="979" uniqueCount="532">
   <si>
     <t>CEDULA</t>
   </si>
@@ -2835,6 +2929,9 @@
   </si>
   <si>
     <t>miercoles</t>
+  </si>
+  <si>
+    <t>carnet</t>
   </si>
 </sst>
 </file>
@@ -2856,7 +2953,7 @@
     <numFmt numFmtId="175" formatCode="#0.0#%"/>
     <numFmt numFmtId="176" formatCode="0.0#"/>
   </numFmts>
-  <fonts count="36">
+  <fonts count="37">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -3073,6 +3170,14 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="18">
@@ -3791,7 +3896,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="181">
+  <cellXfs count="182">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -4111,6 +4216,19 @@
     <xf numFmtId="171" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="175" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="25" fillId="17" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="16" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -4135,24 +4253,16 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="25" fillId="17" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="25" fillId="16" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -13491,14 +13601,14 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:AB37"/>
+  <dimension ref="A1:AC37"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="4" width="16" customWidth="1"/>
-    <col min="5" max="28" width="9" customWidth="1"/>
+    <col min="1" max="5" width="16" customWidth="1"/>
+    <col min="6" max="29" width="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28">
+    <row r="1" spans="1:29">
       <c r="A1" t="s">
         <v>508</v>
       </c>
@@ -13506,7 +13616,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="2" spans="1:28">
+    <row r="2" spans="1:29">
       <c r="A2" t="s">
         <v>509</v>
       </c>
@@ -13514,7 +13624,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="3" spans="1:28">
+    <row r="3" spans="1:29">
       <c r="A3" t="s">
         <v>510</v>
       </c>
@@ -13522,7 +13632,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:28">
+    <row r="5" spans="1:29">
       <c r="A5" s="165" t="s">
         <v>511</v>
       </c>
@@ -13535,1380 +13645,1475 @@
       <c r="D5" s="165" t="s">
         <v>514</v>
       </c>
-      <c r="E5" s="165" t="s">
+      <c r="E5" s="181" t="s">
+        <v>531</v>
+      </c>
+      <c r="F5" s="165" t="s">
         <v>515</v>
       </c>
-      <c r="F5" s="165"/>
-      <c r="G5" s="165" t="s">
+      <c r="G5" s="165"/>
+      <c r="H5" s="165" t="s">
         <v>516</v>
       </c>
-      <c r="H5" s="165"/>
-      <c r="I5" s="165" t="s">
+      <c r="I5" s="165"/>
+      <c r="J5" s="165" t="s">
         <v>517</v>
       </c>
-      <c r="J5" s="165"/>
-      <c r="K5" s="165" t="s">
+      <c r="K5" s="165"/>
+      <c r="L5" s="165" t="s">
         <v>518</v>
       </c>
-      <c r="L5" s="165"/>
-      <c r="M5" s="165" t="s">
+      <c r="M5" s="165"/>
+      <c r="N5" s="165" t="s">
         <v>519</v>
       </c>
-      <c r="N5" s="165"/>
-      <c r="O5" s="165" t="s">
+      <c r="O5" s="165"/>
+      <c r="P5" s="165" t="s">
         <v>520</v>
       </c>
-      <c r="P5" s="165"/>
-      <c r="Q5" s="165" t="s">
+      <c r="Q5" s="165"/>
+      <c r="R5" s="165" t="s">
         <v>521</v>
       </c>
-      <c r="R5" s="165"/>
-      <c r="S5" s="165" t="s">
+      <c r="S5" s="165"/>
+      <c r="T5" s="165" t="s">
         <v>522</v>
       </c>
-      <c r="T5" s="165"/>
-      <c r="U5" s="165" t="s">
+      <c r="U5" s="165"/>
+      <c r="V5" s="165" t="s">
         <v>523</v>
       </c>
-      <c r="V5" s="165"/>
-      <c r="W5" s="165" t="s">
+      <c r="W5" s="165"/>
+      <c r="X5" s="165" t="s">
         <v>524</v>
       </c>
-      <c r="X5" s="165"/>
-      <c r="Y5" s="165" t="s">
+      <c r="Y5" s="165"/>
+      <c r="Z5" s="165" t="s">
         <v>525</v>
       </c>
-      <c r="Z5" s="165"/>
-      <c r="AA5" s="165" t="s">
+      <c r="AA5" s="165"/>
+      <c r="AB5" s="165" t="s">
         <v>526</v>
       </c>
-      <c r="AB5" s="165"/>
-    </row>
-    <row r="6" spans="1:28">
+      <c r="AC5" s="165"/>
+    </row>
+    <row r="6" spans="1:29">
       <c r="A6" s="165"/>
       <c r="B6" s="165"/>
       <c r="C6" s="165"/>
       <c r="D6" s="165"/>
-      <c r="E6" s="130" t="s">
+      <c r="E6" s="180"/>
+      <c r="F6" s="130" t="s">
         <v>529</v>
       </c>
-      <c r="F6" s="130" t="s">
+      <c r="G6" s="130" t="s">
         <v>530</v>
       </c>
-      <c r="G6" s="130" t="s">
+      <c r="H6" s="130" t="s">
         <v>529</v>
       </c>
-      <c r="H6" s="130" t="s">
+      <c r="I6" s="130" t="s">
         <v>530</v>
       </c>
-      <c r="I6" s="130" t="s">
+      <c r="J6" s="130" t="s">
         <v>529</v>
       </c>
-      <c r="J6" s="130" t="s">
+      <c r="K6" s="130" t="s">
         <v>530</v>
       </c>
-      <c r="K6" s="130" t="s">
+      <c r="L6" s="130" t="s">
         <v>529</v>
       </c>
-      <c r="L6" s="130" t="s">
+      <c r="M6" s="130" t="s">
         <v>530</v>
       </c>
-      <c r="M6" s="130" t="s">
+      <c r="N6" s="130" t="s">
         <v>529</v>
       </c>
-      <c r="N6" s="130" t="s">
+      <c r="O6" s="130" t="s">
         <v>530</v>
       </c>
-      <c r="O6" s="130" t="s">
+      <c r="P6" s="130" t="s">
         <v>529</v>
       </c>
-      <c r="P6" s="130" t="s">
+      <c r="Q6" s="130" t="s">
         <v>530</v>
       </c>
-      <c r="Q6" s="130" t="s">
+      <c r="R6" s="130" t="s">
         <v>529</v>
       </c>
-      <c r="R6" s="130" t="s">
+      <c r="S6" s="130" t="s">
         <v>530</v>
       </c>
-      <c r="S6" s="130" t="s">
+      <c r="T6" s="130" t="s">
         <v>529</v>
       </c>
-      <c r="T6" s="130" t="s">
+      <c r="U6" s="130" t="s">
         <v>530</v>
       </c>
-      <c r="U6" s="130" t="s">
+      <c r="V6" s="130" t="s">
         <v>529</v>
       </c>
-      <c r="V6" s="130" t="s">
+      <c r="W6" s="130" t="s">
         <v>530</v>
       </c>
-      <c r="W6" s="130" t="s">
+      <c r="X6" s="130" t="s">
         <v>529</v>
       </c>
-      <c r="X6" s="130" t="s">
+      <c r="Y6" s="130" t="s">
         <v>530</v>
       </c>
-      <c r="Y6" s="130" t="s">
+      <c r="Z6" s="130" t="s">
         <v>529</v>
       </c>
-      <c r="Z6" s="130" t="s">
+      <c r="AA6" s="130" t="s">
         <v>530</v>
       </c>
-      <c r="AA6" s="130" t="s">
+      <c r="AB6" s="130" t="s">
         <v>529</v>
       </c>
-      <c r="AB6" s="130" t="s">
+      <c r="AC6" s="130" t="s">
         <v>530</v>
       </c>
     </row>
-    <row r="7" spans="1:28">
-      <c r="A7" s="168">
-        <v>1</v>
-      </c>
-      <c r="B7" s="170" t="s">
+    <row r="7" spans="1:29">
+      <c r="A7" s="153">
+        <v>1</v>
+      </c>
+      <c r="B7" s="155" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="170" t="s">
+      <c r="C7" s="155" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="168">
+      <c r="D7" s="153">
         <v>30612256</v>
       </c>
-      <c r="E7" s="172">
-        <v>1</v>
-      </c>
-      <c r="F7" s="176"/>
-      <c r="G7" s="172"/>
-      <c r="H7" s="172">
-        <v>1</v>
-      </c>
-      <c r="I7" s="172"/>
-      <c r="J7" s="172"/>
-      <c r="K7" s="172"/>
-      <c r="L7" s="172"/>
-      <c r="N7" s="172"/>
-      <c r="P7" s="172"/>
-      <c r="Q7" s="172"/>
-      <c r="R7" s="172"/>
-      <c r="S7" s="174"/>
-      <c r="T7" s="174"/>
-      <c r="W7" s="174"/>
-      <c r="X7" s="174"/>
-    </row>
-    <row r="8" spans="1:28">
-      <c r="A8" s="169">
+      <c r="E7" s="26">
+        <v>20251110551</v>
+      </c>
+      <c r="F7" s="157">
+        <v>1</v>
+      </c>
+      <c r="G7" s="160"/>
+      <c r="H7" s="157"/>
+      <c r="I7" s="157">
+        <v>1</v>
+      </c>
+      <c r="J7" s="157"/>
+      <c r="K7" s="157"/>
+      <c r="L7" s="157"/>
+      <c r="M7" s="157"/>
+      <c r="O7" s="157"/>
+      <c r="Q7" s="157"/>
+      <c r="R7" s="157"/>
+      <c r="S7" s="157"/>
+      <c r="T7" s="159"/>
+      <c r="U7" s="159"/>
+      <c r="X7" s="159"/>
+      <c r="Y7" s="159"/>
+    </row>
+    <row r="8" spans="1:29">
+      <c r="A8" s="154">
         <v>2</v>
       </c>
-      <c r="B8" s="171" t="s">
+      <c r="B8" s="156" t="s">
         <v>23</v>
       </c>
-      <c r="C8" s="171" t="s">
+      <c r="C8" s="156" t="s">
         <v>22</v>
       </c>
-      <c r="D8" s="169">
+      <c r="D8" s="154">
         <v>31985209</v>
       </c>
-      <c r="E8" s="173"/>
-      <c r="F8" s="177"/>
-      <c r="G8" s="173"/>
-      <c r="H8" s="173"/>
-      <c r="I8" s="173"/>
-      <c r="J8" s="173"/>
-      <c r="K8" s="173"/>
-      <c r="L8" s="173"/>
-      <c r="N8" s="173"/>
-      <c r="P8" s="173"/>
-      <c r="Q8" s="173"/>
-      <c r="R8" s="173"/>
-      <c r="S8" s="180"/>
-      <c r="T8" s="180"/>
-      <c r="W8" s="180"/>
-      <c r="X8" s="180">
+      <c r="E8" s="26">
+        <v>20251110234</v>
+      </c>
+      <c r="F8" s="158"/>
+      <c r="G8" s="161"/>
+      <c r="H8" s="158"/>
+      <c r="I8" s="158"/>
+      <c r="J8" s="158"/>
+      <c r="K8" s="158"/>
+      <c r="L8" s="158"/>
+      <c r="M8" s="158"/>
+      <c r="O8" s="158"/>
+      <c r="Q8" s="158"/>
+      <c r="R8" s="158"/>
+      <c r="S8" s="158"/>
+      <c r="T8" s="164"/>
+      <c r="U8" s="164"/>
+      <c r="X8" s="164"/>
+      <c r="Y8" s="164">
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:28">
-      <c r="A9" s="168">
+    <row r="9" spans="1:29">
+      <c r="A9" s="153">
         <v>3</v>
       </c>
-      <c r="B9" s="170" t="s">
+      <c r="B9" s="155" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="170" t="s">
+      <c r="C9" s="155" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="168">
+      <c r="D9" s="153">
         <v>27670956</v>
       </c>
-      <c r="E9" s="172"/>
-      <c r="F9" s="176"/>
-      <c r="G9" s="172">
+      <c r="E9" s="26">
+        <v>20251110197</v>
+      </c>
+      <c r="F9" s="157"/>
+      <c r="G9" s="160"/>
+      <c r="H9" s="157">
         <v>2</v>
       </c>
-      <c r="H9" s="172"/>
-      <c r="I9" s="172">
-        <v>1</v>
-      </c>
-      <c r="J9" s="172">
-        <v>1</v>
-      </c>
-      <c r="K9" s="172"/>
-      <c r="L9" s="172">
+      <c r="I9" s="157"/>
+      <c r="J9" s="157">
+        <v>1</v>
+      </c>
+      <c r="K9" s="157">
+        <v>1</v>
+      </c>
+      <c r="L9" s="157"/>
+      <c r="M9" s="157">
         <v>2</v>
       </c>
-      <c r="N9" s="172">
-        <v>1</v>
-      </c>
-      <c r="P9" s="172">
+      <c r="O9" s="157">
+        <v>1</v>
+      </c>
+      <c r="Q9" s="157">
         <v>2</v>
       </c>
-      <c r="Q9" s="172">
-        <v>1</v>
-      </c>
-      <c r="R9" s="172">
-        <v>1</v>
-      </c>
-      <c r="S9" s="172">
+      <c r="R9" s="157">
+        <v>1</v>
+      </c>
+      <c r="S9" s="157">
+        <v>1</v>
+      </c>
+      <c r="T9" s="157">
         <v>3</v>
       </c>
-      <c r="T9" s="174">
-        <v>1</v>
-      </c>
-      <c r="W9" s="174">
-        <v>1</v>
-      </c>
-      <c r="X9" s="174">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:28">
-      <c r="A10" s="168">
+      <c r="U9" s="159">
+        <v>1</v>
+      </c>
+      <c r="X9" s="159">
+        <v>1</v>
+      </c>
+      <c r="Y9" s="159">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:29">
+      <c r="A10" s="153">
         <v>4</v>
       </c>
-      <c r="B10" s="171" t="s">
+      <c r="B10" s="156" t="s">
         <v>31</v>
       </c>
-      <c r="C10" s="171" t="s">
+      <c r="C10" s="156" t="s">
         <v>30</v>
       </c>
-      <c r="D10" s="169">
+      <c r="D10" s="154">
         <v>32241977</v>
       </c>
-      <c r="E10" s="173"/>
-      <c r="F10" s="177">
+      <c r="E10" s="26">
+        <v>20251110154</v>
+      </c>
+      <c r="F10" s="158"/>
+      <c r="G10" s="161">
         <v>2</v>
       </c>
-      <c r="G10" s="173"/>
-      <c r="H10" s="173"/>
-      <c r="I10" s="173"/>
-      <c r="J10" s="173"/>
-      <c r="K10" s="173"/>
-      <c r="L10" s="173"/>
-      <c r="N10" s="173"/>
-      <c r="P10" s="173"/>
-      <c r="Q10" s="173"/>
-      <c r="R10" s="173"/>
-      <c r="S10" s="180"/>
-      <c r="T10" s="180"/>
-      <c r="W10" s="180"/>
-      <c r="X10" s="180"/>
-    </row>
-    <row r="11" spans="1:28">
-      <c r="A11" s="169">
+      <c r="H10" s="158"/>
+      <c r="I10" s="158"/>
+      <c r="J10" s="158"/>
+      <c r="K10" s="158"/>
+      <c r="L10" s="158"/>
+      <c r="M10" s="158"/>
+      <c r="O10" s="158"/>
+      <c r="Q10" s="158"/>
+      <c r="R10" s="158"/>
+      <c r="S10" s="158"/>
+      <c r="T10" s="164"/>
+      <c r="U10" s="164"/>
+      <c r="X10" s="164"/>
+      <c r="Y10" s="164"/>
+    </row>
+    <row r="11" spans="1:29">
+      <c r="A11" s="154">
         <v>5</v>
       </c>
-      <c r="B11" s="170" t="s">
+      <c r="B11" s="155" t="s">
         <v>35</v>
       </c>
-      <c r="C11" s="170" t="s">
+      <c r="C11" s="155" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="168">
+      <c r="D11" s="153">
         <v>30888238</v>
       </c>
-      <c r="E11" s="172"/>
-      <c r="F11" s="176">
-        <v>1</v>
-      </c>
-      <c r="G11" s="172">
+      <c r="E11" s="26">
+        <v>20251110558</v>
+      </c>
+      <c r="F11" s="157"/>
+      <c r="G11" s="160">
+        <v>1</v>
+      </c>
+      <c r="H11" s="157">
         <v>2</v>
       </c>
-      <c r="H11" s="172"/>
-      <c r="I11" s="172"/>
-      <c r="J11" s="172"/>
-      <c r="K11" s="172"/>
-      <c r="L11" s="172">
+      <c r="I11" s="157"/>
+      <c r="J11" s="157"/>
+      <c r="K11" s="157"/>
+      <c r="L11" s="157"/>
+      <c r="M11" s="157">
         <v>4</v>
       </c>
-      <c r="N11" s="172">
-        <v>1</v>
-      </c>
-      <c r="P11" s="172">
-        <v>1</v>
-      </c>
-      <c r="Q11" s="172">
-        <v>1</v>
-      </c>
-      <c r="R11" s="172"/>
-      <c r="S11" s="174"/>
-      <c r="T11" s="174"/>
-      <c r="W11" s="174"/>
-      <c r="X11" s="174"/>
-    </row>
-    <row r="12" spans="1:28">
-      <c r="A12" s="168">
+      <c r="O11" s="157">
+        <v>1</v>
+      </c>
+      <c r="Q11" s="157">
+        <v>1</v>
+      </c>
+      <c r="R11" s="157">
+        <v>1</v>
+      </c>
+      <c r="S11" s="157"/>
+      <c r="T11" s="159"/>
+      <c r="U11" s="159"/>
+      <c r="X11" s="159"/>
+      <c r="Y11" s="159"/>
+    </row>
+    <row r="12" spans="1:29">
+      <c r="A12" s="153">
         <v>6</v>
       </c>
-      <c r="B12" s="171" t="s">
+      <c r="B12" s="156" t="s">
         <v>40</v>
       </c>
-      <c r="C12" s="171" t="s">
+      <c r="C12" s="156" t="s">
         <v>39</v>
       </c>
-      <c r="D12" s="169">
+      <c r="D12" s="154">
         <v>30539028</v>
       </c>
-      <c r="E12" s="173"/>
-      <c r="F12" s="177"/>
-      <c r="G12" s="173"/>
-      <c r="H12" s="173"/>
-      <c r="I12" s="173"/>
-      <c r="J12" s="173"/>
-      <c r="K12" s="173"/>
-      <c r="L12" s="173"/>
-      <c r="N12" s="173"/>
-      <c r="P12" s="173"/>
-      <c r="Q12" s="173"/>
-      <c r="R12" s="173"/>
-      <c r="S12" s="180"/>
-      <c r="T12" s="180"/>
-      <c r="W12" s="180"/>
-      <c r="X12" s="180"/>
-    </row>
-    <row r="13" spans="1:28">
-      <c r="A13" s="168">
+      <c r="E12" s="26">
+        <v>20251110300</v>
+      </c>
+      <c r="F12" s="158"/>
+      <c r="G12" s="161"/>
+      <c r="H12" s="158"/>
+      <c r="I12" s="158"/>
+      <c r="J12" s="158"/>
+      <c r="K12" s="158"/>
+      <c r="L12" s="158"/>
+      <c r="M12" s="158"/>
+      <c r="O12" s="158"/>
+      <c r="Q12" s="158"/>
+      <c r="R12" s="158"/>
+      <c r="S12" s="158"/>
+      <c r="T12" s="164"/>
+      <c r="U12" s="164"/>
+      <c r="X12" s="164"/>
+      <c r="Y12" s="164"/>
+    </row>
+    <row r="13" spans="1:29">
+      <c r="A13" s="153">
         <v>7</v>
       </c>
-      <c r="B13" s="170" t="s">
+      <c r="B13" s="155" t="s">
         <v>44</v>
       </c>
-      <c r="C13" s="170" t="s">
+      <c r="C13" s="155" t="s">
         <v>43</v>
       </c>
-      <c r="D13" s="168">
+      <c r="D13" s="153">
         <v>31423864</v>
       </c>
-      <c r="E13" s="172"/>
-      <c r="F13" s="176"/>
-      <c r="G13" s="172"/>
-      <c r="H13" s="172"/>
-      <c r="I13" s="172"/>
-      <c r="J13" s="172"/>
-      <c r="K13" s="172"/>
-      <c r="L13" s="172"/>
-      <c r="N13" s="172"/>
-      <c r="P13" s="172"/>
-      <c r="Q13" s="172"/>
-      <c r="R13" s="172"/>
-      <c r="S13" s="174"/>
-      <c r="T13" s="174"/>
-      <c r="W13" s="174"/>
-      <c r="X13" s="174"/>
-    </row>
-    <row r="14" spans="1:28">
-      <c r="A14" s="169">
+      <c r="E13" s="26">
+        <v>20251110160</v>
+      </c>
+      <c r="F13" s="157"/>
+      <c r="G13" s="160"/>
+      <c r="H13" s="157"/>
+      <c r="I13" s="157"/>
+      <c r="J13" s="157"/>
+      <c r="K13" s="157"/>
+      <c r="L13" s="157"/>
+      <c r="M13" s="157"/>
+      <c r="O13" s="157"/>
+      <c r="Q13" s="157"/>
+      <c r="R13" s="157"/>
+      <c r="S13" s="157"/>
+      <c r="T13" s="159"/>
+      <c r="U13" s="159"/>
+      <c r="X13" s="159"/>
+      <c r="Y13" s="159"/>
+    </row>
+    <row r="14" spans="1:29">
+      <c r="A14" s="154">
         <v>8</v>
       </c>
-      <c r="B14" s="171" t="s">
+      <c r="B14" s="156" t="s">
         <v>48</v>
       </c>
-      <c r="C14" s="171" t="s">
+      <c r="C14" s="156" t="s">
         <v>47</v>
       </c>
-      <c r="D14" s="169">
+      <c r="D14" s="154">
         <v>31979046</v>
       </c>
-      <c r="E14" s="173"/>
-      <c r="F14" s="177">
+      <c r="E14" s="26">
+        <v>20241130202</v>
+      </c>
+      <c r="F14" s="158"/>
+      <c r="G14" s="161">
         <v>2</v>
       </c>
-      <c r="G14" s="173"/>
-      <c r="H14" s="173"/>
-      <c r="I14" s="173"/>
-      <c r="J14" s="173"/>
-      <c r="K14" s="173"/>
-      <c r="L14" s="173">
+      <c r="H14" s="158"/>
+      <c r="I14" s="158"/>
+      <c r="J14" s="158"/>
+      <c r="K14" s="158"/>
+      <c r="L14" s="158"/>
+      <c r="M14" s="158">
         <v>2</v>
       </c>
-      <c r="N14" s="173"/>
-      <c r="P14" s="173"/>
-      <c r="Q14" s="173"/>
-      <c r="R14" s="173">
-        <v>1</v>
-      </c>
-      <c r="S14" s="180">
-        <v>1</v>
-      </c>
-      <c r="T14" s="180"/>
-      <c r="W14" s="180">
-        <v>1</v>
-      </c>
-      <c r="X14" s="180">
+      <c r="O14" s="158"/>
+      <c r="Q14" s="158"/>
+      <c r="R14" s="158"/>
+      <c r="S14" s="158">
+        <v>1</v>
+      </c>
+      <c r="T14" s="164">
+        <v>1</v>
+      </c>
+      <c r="U14" s="164"/>
+      <c r="X14" s="164">
+        <v>1</v>
+      </c>
+      <c r="Y14" s="164">
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:28">
-      <c r="A15" s="168">
+    <row r="15" spans="1:29">
+      <c r="A15" s="153">
         <v>9</v>
       </c>
-      <c r="B15" s="170" t="s">
+      <c r="B15" s="155" t="s">
         <v>52</v>
       </c>
-      <c r="C15" s="170" t="s">
+      <c r="C15" s="155" t="s">
         <v>51</v>
       </c>
-      <c r="D15" s="168">
+      <c r="D15" s="153">
         <v>32042714</v>
       </c>
-      <c r="E15" s="172"/>
-      <c r="F15" s="176"/>
-      <c r="G15" s="172"/>
-      <c r="H15" s="172"/>
-      <c r="I15" s="172">
+      <c r="E15" s="26">
+        <v>20251110345</v>
+      </c>
+      <c r="F15" s="157"/>
+      <c r="G15" s="160"/>
+      <c r="H15" s="157"/>
+      <c r="I15" s="157"/>
+      <c r="J15" s="157">
         <v>2</v>
       </c>
-      <c r="J15" s="172"/>
-      <c r="K15" s="172">
+      <c r="K15" s="157"/>
+      <c r="L15" s="157">
         <v>2</v>
       </c>
-      <c r="L15" s="172">
-        <v>1</v>
-      </c>
-      <c r="N15" s="172">
-        <v>1</v>
-      </c>
-      <c r="P15" s="172">
-        <v>1</v>
-      </c>
-      <c r="Q15" s="172">
-        <v>1</v>
-      </c>
-      <c r="R15" s="172">
-        <v>1</v>
-      </c>
-      <c r="S15" s="172">
+      <c r="M15" s="157">
+        <v>1</v>
+      </c>
+      <c r="O15" s="157">
+        <v>1</v>
+      </c>
+      <c r="Q15" s="157">
+        <v>1</v>
+      </c>
+      <c r="R15" s="157">
+        <v>1</v>
+      </c>
+      <c r="S15" s="157">
+        <v>1</v>
+      </c>
+      <c r="T15" s="157">
         <v>3</v>
       </c>
-      <c r="T15" s="174">
+      <c r="U15" s="159">
         <v>3</v>
       </c>
-      <c r="W15" s="174">
-        <v>1</v>
-      </c>
-      <c r="X15" s="174"/>
-    </row>
-    <row r="16" spans="1:28">
-      <c r="A16" s="168">
+      <c r="X15" s="159">
+        <v>1</v>
+      </c>
+      <c r="Y15" s="159"/>
+    </row>
+    <row r="16" spans="1:29">
+      <c r="A16" s="153">
         <v>10</v>
       </c>
-      <c r="B16" s="171" t="s">
+      <c r="B16" s="156" t="s">
         <v>56</v>
       </c>
-      <c r="C16" s="171" t="s">
+      <c r="C16" s="156" t="s">
         <v>55</v>
       </c>
-      <c r="D16" s="169">
+      <c r="D16" s="154">
         <v>31696701</v>
       </c>
-      <c r="E16" s="173">
-        <v>1</v>
-      </c>
-      <c r="F16" s="177">
-        <v>1</v>
-      </c>
-      <c r="G16" s="173"/>
-      <c r="H16" s="173">
-        <v>1</v>
-      </c>
-      <c r="I16" s="173">
+      <c r="E16" s="26">
+        <v>20241120056</v>
+      </c>
+      <c r="F16" s="158">
+        <v>1</v>
+      </c>
+      <c r="G16" s="161">
+        <v>1</v>
+      </c>
+      <c r="H16" s="158"/>
+      <c r="I16" s="158">
+        <v>1</v>
+      </c>
+      <c r="J16" s="158">
         <v>3</v>
       </c>
-      <c r="J16" s="173">
-        <v>1</v>
-      </c>
-      <c r="K16" s="173"/>
-      <c r="L16" s="173">
-        <v>1</v>
-      </c>
-      <c r="N16" s="173">
-        <v>1</v>
-      </c>
-      <c r="P16" s="173">
+      <c r="K16" s="158">
+        <v>1</v>
+      </c>
+      <c r="L16" s="158"/>
+      <c r="M16" s="158">
+        <v>1</v>
+      </c>
+      <c r="O16" s="158">
+        <v>1</v>
+      </c>
+      <c r="Q16" s="158">
         <v>3</v>
       </c>
-      <c r="Q16" s="173">
-        <v>1</v>
-      </c>
-      <c r="R16" s="173">
-        <v>1</v>
-      </c>
-      <c r="S16" s="173">
+      <c r="R16" s="158">
+        <v>1</v>
+      </c>
+      <c r="S16" s="158">
+        <v>1</v>
+      </c>
+      <c r="T16" s="158">
         <v>3</v>
       </c>
-      <c r="T16" s="173">
+      <c r="U16" s="158">
         <v>3</v>
       </c>
-      <c r="W16" s="180">
-        <v>1</v>
-      </c>
-      <c r="X16" s="180">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:24">
-      <c r="A17" s="169">
+      <c r="X16" s="164">
+        <v>1</v>
+      </c>
+      <c r="Y16" s="164">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:25">
+      <c r="A17" s="154">
         <v>11</v>
       </c>
-      <c r="B17" s="170" t="s">
+      <c r="B17" s="155" t="s">
         <v>60</v>
       </c>
-      <c r="C17" s="170" t="s">
+      <c r="C17" s="155" t="s">
         <v>59</v>
       </c>
-      <c r="D17" s="168">
+      <c r="D17" s="153">
         <v>31935772</v>
       </c>
-      <c r="E17" s="172"/>
-      <c r="F17" s="176"/>
-      <c r="G17" s="172">
+      <c r="E17" s="26">
+        <v>20241130203</v>
+      </c>
+      <c r="F17" s="157"/>
+      <c r="G17" s="160"/>
+      <c r="H17" s="157">
         <v>2</v>
       </c>
-      <c r="H17" s="172"/>
-      <c r="I17" s="172"/>
-      <c r="J17" s="172"/>
-      <c r="K17" s="172"/>
-      <c r="L17" s="172">
+      <c r="I17" s="157"/>
+      <c r="J17" s="157"/>
+      <c r="K17" s="157"/>
+      <c r="L17" s="157"/>
+      <c r="M17" s="157">
         <v>2</v>
       </c>
-      <c r="N17" s="172">
-        <v>1</v>
-      </c>
-      <c r="P17" s="172"/>
-      <c r="Q17" s="172"/>
-      <c r="R17" s="172">
-        <v>1</v>
-      </c>
-      <c r="S17" s="174"/>
-      <c r="T17" s="174"/>
-      <c r="W17" s="174"/>
-      <c r="X17" s="174"/>
-    </row>
-    <row r="18" spans="1:24">
-      <c r="A18" s="168">
+      <c r="O17" s="157">
+        <v>1</v>
+      </c>
+      <c r="Q17" s="157"/>
+      <c r="R17" s="157"/>
+      <c r="S17" s="157">
+        <v>1</v>
+      </c>
+      <c r="T17" s="159"/>
+      <c r="U17" s="159"/>
+      <c r="X17" s="159"/>
+      <c r="Y17" s="159"/>
+    </row>
+    <row r="18" spans="1:25">
+      <c r="A18" s="153">
         <v>12</v>
       </c>
-      <c r="B18" s="171" t="s">
+      <c r="B18" s="156" t="s">
         <v>64</v>
       </c>
-      <c r="C18" s="171" t="s">
+      <c r="C18" s="156" t="s">
         <v>63</v>
       </c>
-      <c r="D18" s="169">
+      <c r="D18" s="154">
         <v>31886469</v>
       </c>
-      <c r="E18" s="173"/>
-      <c r="F18" s="177"/>
-      <c r="G18" s="173"/>
-      <c r="H18" s="173"/>
-      <c r="I18" s="173"/>
-      <c r="J18" s="173"/>
-      <c r="K18" s="173"/>
-      <c r="L18" s="173"/>
-      <c r="N18" s="173"/>
-      <c r="P18" s="173"/>
-      <c r="Q18" s="173"/>
-      <c r="R18" s="173"/>
-      <c r="S18" s="180"/>
-      <c r="T18" s="180"/>
-      <c r="W18" s="180"/>
-      <c r="X18" s="180"/>
-    </row>
-    <row r="19" spans="1:24">
-      <c r="A19" s="168">
+      <c r="E18" s="26">
+        <v>20251110136</v>
+      </c>
+      <c r="F18" s="158"/>
+      <c r="G18" s="161"/>
+      <c r="H18" s="158"/>
+      <c r="I18" s="158"/>
+      <c r="J18" s="158"/>
+      <c r="K18" s="158"/>
+      <c r="L18" s="158"/>
+      <c r="M18" s="158"/>
+      <c r="O18" s="158"/>
+      <c r="Q18" s="158"/>
+      <c r="R18" s="158"/>
+      <c r="S18" s="158"/>
+      <c r="T18" s="164"/>
+      <c r="U18" s="164"/>
+      <c r="X18" s="164"/>
+      <c r="Y18" s="164"/>
+    </row>
+    <row r="19" spans="1:25">
+      <c r="A19" s="153">
         <v>13</v>
       </c>
-      <c r="B19" s="170" t="s">
+      <c r="B19" s="155" t="s">
         <v>68</v>
       </c>
-      <c r="C19" s="170" t="s">
+      <c r="C19" s="155" t="s">
         <v>67</v>
       </c>
-      <c r="D19" s="168">
+      <c r="D19" s="153">
         <v>32121959</v>
       </c>
-      <c r="E19" s="172"/>
-      <c r="F19" s="176"/>
-      <c r="G19" s="172"/>
-      <c r="H19" s="172"/>
-      <c r="I19" s="172"/>
-      <c r="J19" s="172"/>
-      <c r="K19" s="172"/>
-      <c r="L19" s="172"/>
-      <c r="N19" s="172"/>
-      <c r="P19" s="172"/>
-      <c r="Q19" s="172"/>
-      <c r="R19" s="172"/>
-      <c r="S19" s="174"/>
-      <c r="T19" s="174"/>
-      <c r="W19" s="174"/>
-      <c r="X19" s="174"/>
-    </row>
-    <row r="20" spans="1:24">
-      <c r="A20" s="169">
+      <c r="E19" s="26">
+        <v>20251110391</v>
+      </c>
+      <c r="F19" s="157"/>
+      <c r="G19" s="160"/>
+      <c r="H19" s="157"/>
+      <c r="I19" s="157"/>
+      <c r="J19" s="157"/>
+      <c r="K19" s="157"/>
+      <c r="L19" s="157"/>
+      <c r="M19" s="157"/>
+      <c r="O19" s="157"/>
+      <c r="Q19" s="157"/>
+      <c r="R19" s="157"/>
+      <c r="S19" s="157"/>
+      <c r="T19" s="159"/>
+      <c r="U19" s="159"/>
+      <c r="X19" s="159"/>
+      <c r="Y19" s="159"/>
+    </row>
+    <row r="20" spans="1:25">
+      <c r="A20" s="154">
         <v>14</v>
       </c>
-      <c r="B20" s="171" t="s">
+      <c r="B20" s="156" t="s">
         <v>72</v>
       </c>
-      <c r="C20" s="171" t="s">
+      <c r="C20" s="156" t="s">
         <v>71</v>
       </c>
-      <c r="D20" s="169">
+      <c r="D20" s="154">
         <v>32235827</v>
       </c>
-      <c r="E20" s="173">
+      <c r="E20" s="26">
+        <v>20251110201</v>
+      </c>
+      <c r="F20" s="158">
         <v>3</v>
       </c>
-      <c r="F20" s="177">
+      <c r="G20" s="161">
         <v>3</v>
       </c>
-      <c r="G20" s="173">
+      <c r="H20" s="158">
         <v>3</v>
       </c>
-      <c r="H20" s="173">
+      <c r="I20" s="158">
         <v>2</v>
       </c>
-      <c r="I20" s="173"/>
-      <c r="J20" s="173">
+      <c r="J20" s="158"/>
+      <c r="K20" s="158">
         <v>3</v>
       </c>
-      <c r="K20" s="173"/>
-      <c r="L20" s="173">
-        <v>1</v>
-      </c>
-      <c r="N20" s="173">
-        <v>1</v>
-      </c>
-      <c r="P20" s="173">
-        <v>1</v>
-      </c>
-      <c r="Q20" s="173"/>
-      <c r="R20" s="173">
-        <v>1</v>
-      </c>
-      <c r="S20" s="173">
-        <v>1</v>
-      </c>
-      <c r="T20" s="180">
+      <c r="L20" s="158"/>
+      <c r="M20" s="158">
+        <v>1</v>
+      </c>
+      <c r="O20" s="158">
+        <v>1</v>
+      </c>
+      <c r="Q20" s="158">
+        <v>1</v>
+      </c>
+      <c r="R20" s="158"/>
+      <c r="S20" s="158">
+        <v>1</v>
+      </c>
+      <c r="T20" s="158">
+        <v>1</v>
+      </c>
+      <c r="U20" s="164">
         <v>3</v>
       </c>
-      <c r="W20" s="180">
-        <v>1</v>
-      </c>
-      <c r="X20" s="180"/>
-    </row>
-    <row r="21" spans="1:24">
-      <c r="A21" s="168">
+      <c r="X20" s="164">
+        <v>1</v>
+      </c>
+      <c r="Y20" s="164"/>
+    </row>
+    <row r="21" spans="1:25">
+      <c r="A21" s="153">
         <v>15</v>
       </c>
-      <c r="B21" s="170" t="s">
+      <c r="B21" s="155" t="s">
         <v>76</v>
       </c>
-      <c r="C21" s="170" t="s">
+      <c r="C21" s="155" t="s">
         <v>75</v>
       </c>
-      <c r="D21" s="168">
+      <c r="D21" s="153">
         <v>31873119</v>
       </c>
-      <c r="E21" s="172">
-        <v>1</v>
-      </c>
-      <c r="F21" s="176"/>
-      <c r="G21" s="172">
-        <v>1</v>
-      </c>
-      <c r="H21" s="172">
-        <v>1</v>
-      </c>
-      <c r="I21" s="172">
-        <v>1</v>
-      </c>
-      <c r="J21" s="172">
-        <v>1</v>
-      </c>
-      <c r="K21" s="172">
+      <c r="E21" s="26">
+        <v>20251110492</v>
+      </c>
+      <c r="F21" s="157">
+        <v>1</v>
+      </c>
+      <c r="G21" s="160"/>
+      <c r="H21" s="157">
+        <v>1</v>
+      </c>
+      <c r="I21" s="157">
+        <v>1</v>
+      </c>
+      <c r="J21" s="157">
+        <v>1</v>
+      </c>
+      <c r="K21" s="157">
+        <v>1</v>
+      </c>
+      <c r="L21" s="157">
         <v>2</v>
       </c>
-      <c r="L21" s="172">
+      <c r="M21" s="157">
         <v>2</v>
       </c>
-      <c r="N21" s="172">
-        <v>1</v>
-      </c>
-      <c r="P21" s="172">
+      <c r="O21" s="157">
+        <v>1</v>
+      </c>
+      <c r="Q21" s="157">
         <v>2</v>
       </c>
-      <c r="Q21" s="172">
+      <c r="R21" s="157">
         <v>3</v>
       </c>
-      <c r="R21" s="172">
-        <v>1</v>
-      </c>
-      <c r="S21" s="174">
+      <c r="S21" s="157">
+        <v>1</v>
+      </c>
+      <c r="T21" s="159">
         <v>3</v>
       </c>
-      <c r="T21" s="174">
+      <c r="U21" s="159">
         <v>3</v>
       </c>
-      <c r="W21" s="174">
-        <v>1</v>
-      </c>
-      <c r="X21" s="174">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:24">
-      <c r="A22" s="168">
+      <c r="X21" s="159">
+        <v>1</v>
+      </c>
+      <c r="Y21" s="159">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:25">
+      <c r="A22" s="153">
         <v>16</v>
       </c>
-      <c r="B22" s="171" t="s">
+      <c r="B22" s="156" t="s">
         <v>80</v>
       </c>
-      <c r="C22" s="171" t="s">
+      <c r="C22" s="156" t="s">
         <v>79</v>
       </c>
-      <c r="D22" s="169">
+      <c r="D22" s="154">
         <v>27007813</v>
       </c>
-      <c r="E22" s="173"/>
-      <c r="F22" s="177"/>
-      <c r="G22" s="173"/>
-      <c r="H22" s="173"/>
-      <c r="I22" s="173"/>
-      <c r="J22" s="173"/>
-      <c r="K22" s="173"/>
-      <c r="L22" s="173"/>
-      <c r="N22" s="173"/>
-      <c r="P22" s="173"/>
-      <c r="Q22" s="173"/>
-      <c r="R22" s="173">
-        <v>1</v>
-      </c>
-      <c r="S22" s="180"/>
-      <c r="T22" s="180"/>
-      <c r="W22" s="180"/>
-      <c r="X22" s="180"/>
-    </row>
-    <row r="23" spans="1:24">
-      <c r="A23" s="169">
+      <c r="E22" s="26">
+        <v>20191110764</v>
+      </c>
+      <c r="F22" s="158"/>
+      <c r="G22" s="161"/>
+      <c r="H22" s="158"/>
+      <c r="I22" s="158"/>
+      <c r="J22" s="158"/>
+      <c r="K22" s="158"/>
+      <c r="L22" s="158"/>
+      <c r="M22" s="158"/>
+      <c r="O22" s="158"/>
+      <c r="Q22" s="158"/>
+      <c r="R22" s="158"/>
+      <c r="S22" s="158">
+        <v>1</v>
+      </c>
+      <c r="T22" s="164"/>
+      <c r="U22" s="164"/>
+      <c r="X22" s="164"/>
+      <c r="Y22" s="164"/>
+    </row>
+    <row r="23" spans="1:25">
+      <c r="A23" s="154">
         <v>17</v>
       </c>
-      <c r="B23" s="170" t="s">
+      <c r="B23" s="155" t="s">
         <v>84</v>
       </c>
-      <c r="C23" s="170" t="s">
+      <c r="C23" s="155" t="s">
         <v>83</v>
       </c>
-      <c r="D23" s="168">
+      <c r="D23" s="153">
         <v>31460623</v>
       </c>
-      <c r="E23" s="172"/>
-      <c r="F23" s="176"/>
-      <c r="G23" s="172"/>
-      <c r="H23" s="172"/>
-      <c r="I23" s="172"/>
-      <c r="J23" s="172"/>
-      <c r="K23" s="172"/>
-      <c r="L23" s="172"/>
-      <c r="N23" s="172"/>
-      <c r="P23" s="172"/>
-      <c r="Q23" s="172"/>
-      <c r="R23" s="172">
-        <v>1</v>
-      </c>
-      <c r="S23" s="174"/>
-      <c r="T23" s="174"/>
-      <c r="W23" s="174"/>
-      <c r="X23" s="174"/>
-    </row>
-    <row r="24" spans="1:24">
-      <c r="A24" s="168">
+      <c r="E23" s="26">
+        <v>20251110246</v>
+      </c>
+      <c r="F23" s="157"/>
+      <c r="G23" s="160"/>
+      <c r="H23" s="157"/>
+      <c r="I23" s="157"/>
+      <c r="J23" s="157"/>
+      <c r="K23" s="157"/>
+      <c r="L23" s="157"/>
+      <c r="M23" s="157"/>
+      <c r="O23" s="157"/>
+      <c r="Q23" s="157"/>
+      <c r="R23" s="157"/>
+      <c r="S23" s="157">
+        <v>1</v>
+      </c>
+      <c r="T23" s="159"/>
+      <c r="U23" s="159"/>
+      <c r="X23" s="159"/>
+      <c r="Y23" s="159"/>
+    </row>
+    <row r="24" spans="1:25">
+      <c r="A24" s="153">
         <v>18</v>
       </c>
-      <c r="B24" s="171" t="s">
+      <c r="B24" s="156" t="s">
         <v>88</v>
       </c>
-      <c r="C24" s="171" t="s">
+      <c r="C24" s="156" t="s">
         <v>87</v>
       </c>
-      <c r="D24" s="169">
+      <c r="D24" s="154">
         <v>33186550</v>
       </c>
-      <c r="E24" s="173"/>
-      <c r="F24" s="177"/>
-      <c r="G24" s="173">
-        <v>1</v>
-      </c>
-      <c r="H24" s="173"/>
-      <c r="I24" s="173">
+      <c r="E24" s="26">
+        <v>20251110348</v>
+      </c>
+      <c r="F24" s="158"/>
+      <c r="G24" s="161"/>
+      <c r="H24" s="158">
+        <v>1</v>
+      </c>
+      <c r="I24" s="158"/>
+      <c r="J24" s="158">
         <v>2</v>
       </c>
-      <c r="J24" s="173">
+      <c r="K24" s="158">
         <v>3</v>
       </c>
-      <c r="K24" s="173"/>
-      <c r="L24" s="173"/>
-      <c r="N24" s="173"/>
-      <c r="P24" s="173">
+      <c r="L24" s="158"/>
+      <c r="M24" s="158"/>
+      <c r="O24" s="158"/>
+      <c r="Q24" s="158">
         <v>4</v>
       </c>
-      <c r="Q24" s="173">
-        <v>1</v>
-      </c>
-      <c r="R24" s="173">
+      <c r="R24" s="158">
+        <v>1</v>
+      </c>
+      <c r="S24" s="158">
         <v>3</v>
       </c>
-      <c r="S24" s="180"/>
-      <c r="T24" s="180">
-        <v>1</v>
-      </c>
-      <c r="W24" s="180">
-        <v>1</v>
-      </c>
-      <c r="X24" s="180">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:24">
-      <c r="A25" s="168">
+      <c r="T24" s="164"/>
+      <c r="U24" s="164">
+        <v>1</v>
+      </c>
+      <c r="X24" s="164">
+        <v>1</v>
+      </c>
+      <c r="Y24" s="164">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:25">
+      <c r="A25" s="153">
         <v>19</v>
       </c>
-      <c r="B25" s="170" t="s">
+      <c r="B25" s="155" t="s">
         <v>92</v>
       </c>
-      <c r="C25" s="170" t="s">
+      <c r="C25" s="155" t="s">
         <v>91</v>
       </c>
-      <c r="D25" s="168">
+      <c r="D25" s="153">
         <v>33219652</v>
       </c>
-      <c r="E25" s="172"/>
-      <c r="F25" s="176"/>
-      <c r="G25" s="172"/>
-      <c r="H25" s="172"/>
-      <c r="I25" s="172"/>
-      <c r="J25" s="172"/>
-      <c r="K25" s="172"/>
-      <c r="L25" s="172"/>
-      <c r="N25" s="172"/>
-      <c r="P25" s="172"/>
-      <c r="Q25" s="172"/>
-      <c r="R25" s="172"/>
-      <c r="S25" s="174"/>
-      <c r="T25" s="174"/>
-      <c r="W25" s="174"/>
-      <c r="X25" s="174"/>
-    </row>
-    <row r="26" spans="1:24">
-      <c r="A26" s="169">
+      <c r="E25" s="26">
+        <v>20251110296</v>
+      </c>
+      <c r="F25" s="157"/>
+      <c r="G25" s="160"/>
+      <c r="H25" s="157"/>
+      <c r="I25" s="157"/>
+      <c r="J25" s="157"/>
+      <c r="K25" s="157"/>
+      <c r="L25" s="157"/>
+      <c r="M25" s="157"/>
+      <c r="O25" s="157"/>
+      <c r="Q25" s="157"/>
+      <c r="R25" s="157"/>
+      <c r="S25" s="157"/>
+      <c r="T25" s="159"/>
+      <c r="U25" s="159"/>
+      <c r="X25" s="159"/>
+      <c r="Y25" s="159"/>
+    </row>
+    <row r="26" spans="1:25">
+      <c r="A26" s="154">
         <v>20</v>
       </c>
-      <c r="B26" s="171" t="s">
+      <c r="B26" s="156" t="s">
         <v>96</v>
       </c>
-      <c r="C26" s="171" t="s">
+      <c r="C26" s="156" t="s">
         <v>95</v>
       </c>
-      <c r="D26" s="169">
+      <c r="D26" s="154">
         <v>31935917</v>
       </c>
-      <c r="E26" s="173"/>
-      <c r="F26" s="177">
-        <v>1</v>
-      </c>
-      <c r="G26" s="178">
+      <c r="E26" s="26">
+        <v>20241130163</v>
+      </c>
+      <c r="F26" s="158"/>
+      <c r="G26" s="161">
+        <v>1</v>
+      </c>
+      <c r="H26" s="162">
         <v>2</v>
       </c>
-      <c r="H26" s="173"/>
-      <c r="I26" s="173">
-        <v>1</v>
-      </c>
-      <c r="J26" s="173"/>
-      <c r="K26" s="173"/>
-      <c r="L26" s="173"/>
-      <c r="N26" s="173"/>
-      <c r="P26" s="173"/>
-      <c r="Q26" s="173"/>
-      <c r="R26" s="173"/>
-      <c r="S26" s="180"/>
-      <c r="T26" s="180"/>
-      <c r="W26" s="180"/>
-      <c r="X26" s="180"/>
-    </row>
-    <row r="27" spans="1:24">
-      <c r="A27" s="168">
+      <c r="I26" s="158"/>
+      <c r="J26" s="158">
+        <v>1</v>
+      </c>
+      <c r="K26" s="158"/>
+      <c r="L26" s="158"/>
+      <c r="M26" s="158"/>
+      <c r="O26" s="158"/>
+      <c r="Q26" s="158"/>
+      <c r="R26" s="158"/>
+      <c r="S26" s="158"/>
+      <c r="T26" s="164"/>
+      <c r="U26" s="164"/>
+      <c r="X26" s="164"/>
+      <c r="Y26" s="164"/>
+    </row>
+    <row r="27" spans="1:25">
+      <c r="A27" s="153">
         <v>21</v>
       </c>
-      <c r="B27" s="170" t="s">
+      <c r="B27" s="155" t="s">
         <v>100</v>
       </c>
-      <c r="C27" s="170" t="s">
+      <c r="C27" s="155" t="s">
         <v>99</v>
       </c>
-      <c r="D27" s="168">
+      <c r="D27" s="153">
         <v>31745168</v>
       </c>
-      <c r="E27" s="172"/>
-      <c r="F27" s="176"/>
-      <c r="G27" s="172"/>
-      <c r="H27" s="172"/>
-      <c r="I27" s="172"/>
-      <c r="J27" s="172"/>
-      <c r="K27" s="172"/>
-      <c r="L27" s="172"/>
-      <c r="N27" s="172">
-        <v>1</v>
-      </c>
-      <c r="P27" s="172">
-        <v>1</v>
-      </c>
-      <c r="Q27" s="172"/>
-      <c r="R27" s="172"/>
-      <c r="S27" s="174"/>
-      <c r="T27" s="174"/>
-      <c r="W27" s="174"/>
-      <c r="X27" s="174"/>
-    </row>
-    <row r="28" spans="1:24">
-      <c r="A28" s="168">
+      <c r="E27" s="26">
+        <v>20251110259</v>
+      </c>
+      <c r="F27" s="157"/>
+      <c r="G27" s="160"/>
+      <c r="H27" s="157"/>
+      <c r="I27" s="157"/>
+      <c r="J27" s="157"/>
+      <c r="K27" s="157"/>
+      <c r="L27" s="157"/>
+      <c r="M27" s="157"/>
+      <c r="O27" s="157">
+        <v>1</v>
+      </c>
+      <c r="Q27" s="157">
+        <v>1</v>
+      </c>
+      <c r="R27" s="157"/>
+      <c r="S27" s="157"/>
+      <c r="T27" s="159"/>
+      <c r="U27" s="159"/>
+      <c r="X27" s="159"/>
+      <c r="Y27" s="159"/>
+    </row>
+    <row r="28" spans="1:25">
+      <c r="A28" s="153">
         <v>22</v>
       </c>
-      <c r="B28" s="171" t="s">
+      <c r="B28" s="156" t="s">
         <v>104</v>
       </c>
-      <c r="C28" s="171" t="s">
+      <c r="C28" s="156" t="s">
         <v>103</v>
       </c>
-      <c r="D28" s="169">
+      <c r="D28" s="154">
         <v>32511604</v>
       </c>
-      <c r="E28" s="173">
+      <c r="E28" s="26">
+        <v>20251110113</v>
+      </c>
+      <c r="F28" s="158">
         <v>2</v>
       </c>
-      <c r="F28" s="177">
+      <c r="G28" s="161">
         <v>2</v>
       </c>
-      <c r="G28" s="173">
-        <v>1</v>
-      </c>
-      <c r="H28" s="173">
-        <v>1</v>
-      </c>
-      <c r="I28" s="173">
-        <v>1</v>
-      </c>
-      <c r="J28" s="173">
-        <v>1</v>
-      </c>
-      <c r="K28" s="173">
+      <c r="H28" s="158">
+        <v>1</v>
+      </c>
+      <c r="I28" s="158">
+        <v>1</v>
+      </c>
+      <c r="J28" s="158">
+        <v>1</v>
+      </c>
+      <c r="K28" s="158">
+        <v>1</v>
+      </c>
+      <c r="L28" s="158">
         <v>3</v>
       </c>
-      <c r="L28" s="173"/>
-      <c r="N28" s="173">
-        <v>1</v>
-      </c>
-      <c r="P28" s="173">
+      <c r="M28" s="158"/>
+      <c r="O28" s="158">
+        <v>1</v>
+      </c>
+      <c r="Q28" s="158">
         <v>2</v>
       </c>
-      <c r="Q28" s="173">
+      <c r="R28" s="158">
         <v>3</v>
       </c>
-      <c r="R28" s="173">
+      <c r="S28" s="158">
         <v>3</v>
       </c>
-      <c r="S28" s="180">
-        <v>1</v>
-      </c>
-      <c r="T28" s="180">
-        <v>1</v>
-      </c>
-      <c r="W28" s="180">
-        <v>1</v>
-      </c>
-      <c r="X28" s="180">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:24">
-      <c r="A29" s="169">
+      <c r="T28" s="164">
+        <v>1</v>
+      </c>
+      <c r="U28" s="164">
+        <v>1</v>
+      </c>
+      <c r="X28" s="164">
+        <v>1</v>
+      </c>
+      <c r="Y28" s="164">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:25">
+      <c r="A29" s="154">
         <v>23</v>
       </c>
-      <c r="B29" s="170" t="s">
+      <c r="B29" s="155" t="s">
         <v>108</v>
       </c>
-      <c r="C29" s="170" t="s">
+      <c r="C29" s="155" t="s">
         <v>107</v>
       </c>
-      <c r="D29" s="168">
+      <c r="D29" s="153">
         <v>31701229</v>
       </c>
-      <c r="E29" s="172"/>
-      <c r="F29" s="176"/>
-      <c r="G29" s="172">
-        <v>1</v>
-      </c>
-      <c r="H29" s="172">
+      <c r="E29" s="26">
+        <v>20251110487</v>
+      </c>
+      <c r="F29" s="157"/>
+      <c r="G29" s="160"/>
+      <c r="H29" s="157">
+        <v>1</v>
+      </c>
+      <c r="I29" s="157">
         <v>2</v>
       </c>
-      <c r="I29" s="172">
-        <v>1</v>
-      </c>
-      <c r="J29" s="172">
-        <v>1</v>
-      </c>
-      <c r="K29" s="172">
+      <c r="J29" s="157">
+        <v>1</v>
+      </c>
+      <c r="K29" s="157">
+        <v>1</v>
+      </c>
+      <c r="L29" s="157">
         <v>3</v>
       </c>
-      <c r="L29" s="172">
+      <c r="M29" s="157">
         <v>3</v>
       </c>
-      <c r="N29" s="172">
+      <c r="O29" s="157">
         <v>3</v>
       </c>
-      <c r="P29" s="172">
-        <v>1</v>
-      </c>
-      <c r="Q29" s="172"/>
-      <c r="R29" s="172">
-        <v>1</v>
-      </c>
-      <c r="S29" s="174">
+      <c r="Q29" s="157">
+        <v>1</v>
+      </c>
+      <c r="R29" s="157"/>
+      <c r="S29" s="157">
+        <v>1</v>
+      </c>
+      <c r="T29" s="159">
         <v>2</v>
       </c>
-      <c r="T29" s="174"/>
-      <c r="W29" s="174">
-        <v>1</v>
-      </c>
-      <c r="X29" s="174"/>
-    </row>
-    <row r="30" spans="1:24">
-      <c r="A30" s="168">
+      <c r="U29" s="159"/>
+      <c r="X29" s="159">
+        <v>1</v>
+      </c>
+      <c r="Y29" s="159"/>
+    </row>
+    <row r="30" spans="1:25">
+      <c r="A30" s="153">
         <v>24</v>
       </c>
-      <c r="B30" s="171" t="s">
+      <c r="B30" s="156" t="s">
         <v>112</v>
       </c>
-      <c r="C30" s="171" t="s">
+      <c r="C30" s="156" t="s">
         <v>111</v>
       </c>
-      <c r="D30" s="169">
+      <c r="D30" s="154">
         <v>30538673</v>
       </c>
-      <c r="E30" s="173">
+      <c r="E30" s="26">
+        <v>20241130215</v>
+      </c>
+      <c r="F30" s="158">
         <v>2</v>
       </c>
-      <c r="F30" s="177"/>
-      <c r="G30" s="173">
-        <v>1</v>
-      </c>
-      <c r="H30" s="173"/>
-      <c r="I30" s="173"/>
-      <c r="J30" s="173">
-        <v>1</v>
-      </c>
-      <c r="K30" s="173"/>
-      <c r="L30" s="173"/>
-      <c r="N30" s="173">
-        <v>1</v>
-      </c>
-      <c r="P30" s="173">
-        <v>1</v>
-      </c>
-      <c r="Q30" s="173"/>
-      <c r="R30" s="173"/>
-      <c r="S30" s="180"/>
-      <c r="T30" s="180"/>
-      <c r="W30" s="180">
-        <v>1</v>
-      </c>
-      <c r="X30" s="180"/>
-    </row>
-    <row r="31" spans="1:24">
-      <c r="A31" s="168">
+      <c r="G30" s="161"/>
+      <c r="H30" s="158">
+        <v>1</v>
+      </c>
+      <c r="I30" s="158"/>
+      <c r="J30" s="158"/>
+      <c r="K30" s="158">
+        <v>1</v>
+      </c>
+      <c r="L30" s="158"/>
+      <c r="M30" s="158"/>
+      <c r="O30" s="158">
+        <v>1</v>
+      </c>
+      <c r="Q30" s="158">
+        <v>1</v>
+      </c>
+      <c r="R30" s="158"/>
+      <c r="S30" s="158"/>
+      <c r="T30" s="164"/>
+      <c r="U30" s="164"/>
+      <c r="X30" s="164">
+        <v>1</v>
+      </c>
+      <c r="Y30" s="164"/>
+    </row>
+    <row r="31" spans="1:25">
+      <c r="A31" s="153">
         <v>25</v>
       </c>
-      <c r="B31" s="170" t="s">
+      <c r="B31" s="155" t="s">
         <v>116</v>
       </c>
-      <c r="C31" s="170" t="s">
+      <c r="C31" s="155" t="s">
         <v>115</v>
       </c>
-      <c r="D31" s="168">
+      <c r="D31" s="153">
         <v>32001850</v>
       </c>
-      <c r="E31" s="172">
+      <c r="E31" s="26">
+        <v>20251110406</v>
+      </c>
+      <c r="F31" s="157">
         <v>2</v>
       </c>
-      <c r="F31" s="176">
-        <v>1</v>
-      </c>
-      <c r="G31" s="172"/>
-      <c r="H31" s="172"/>
-      <c r="I31" s="172"/>
-      <c r="J31" s="172"/>
-      <c r="K31" s="172"/>
-      <c r="L31" s="172">
+      <c r="G31" s="160">
+        <v>1</v>
+      </c>
+      <c r="H31" s="157"/>
+      <c r="I31" s="157"/>
+      <c r="J31" s="157"/>
+      <c r="K31" s="157"/>
+      <c r="L31" s="157"/>
+      <c r="M31" s="157">
         <v>2</v>
       </c>
-      <c r="N31" s="172"/>
-      <c r="P31" s="172"/>
-      <c r="Q31" s="172"/>
-      <c r="R31" s="172"/>
-      <c r="S31" s="174"/>
-      <c r="T31" s="174"/>
-      <c r="W31" s="174"/>
-      <c r="X31" s="174"/>
-    </row>
-    <row r="32" spans="1:24">
-      <c r="A32" s="169">
+      <c r="O31" s="157"/>
+      <c r="Q31" s="157"/>
+      <c r="R31" s="157"/>
+      <c r="S31" s="157"/>
+      <c r="T31" s="159"/>
+      <c r="U31" s="159"/>
+      <c r="X31" s="159"/>
+      <c r="Y31" s="159"/>
+    </row>
+    <row r="32" spans="1:25">
+      <c r="A32" s="154">
         <v>26</v>
       </c>
-      <c r="B32" s="171" t="s">
+      <c r="B32" s="156" t="s">
         <v>120</v>
       </c>
-      <c r="C32" s="171" t="s">
+      <c r="C32" s="156" t="s">
         <v>119</v>
       </c>
-      <c r="D32" s="169">
+      <c r="D32" s="154">
         <v>31873242</v>
       </c>
-      <c r="E32" s="173"/>
-      <c r="F32" s="177"/>
-      <c r="G32" s="173"/>
-      <c r="H32" s="173"/>
-      <c r="I32" s="173"/>
-      <c r="J32" s="173"/>
-      <c r="K32" s="173"/>
-      <c r="L32" s="173"/>
-      <c r="N32" s="173"/>
-      <c r="P32" s="173"/>
-      <c r="Q32" s="173"/>
-      <c r="R32" s="173"/>
-      <c r="S32" s="180"/>
-      <c r="T32" s="180"/>
-      <c r="W32" s="180"/>
-      <c r="X32" s="180"/>
-    </row>
-    <row r="33" spans="1:24">
-      <c r="A33" s="168">
+      <c r="E32" s="26">
+        <v>20251110035</v>
+      </c>
+      <c r="F32" s="158"/>
+      <c r="G32" s="161"/>
+      <c r="H32" s="158"/>
+      <c r="I32" s="158"/>
+      <c r="J32" s="158"/>
+      <c r="K32" s="158"/>
+      <c r="L32" s="158"/>
+      <c r="M32" s="158"/>
+      <c r="O32" s="158"/>
+      <c r="Q32" s="158"/>
+      <c r="R32" s="158"/>
+      <c r="S32" s="158"/>
+      <c r="T32" s="164"/>
+      <c r="U32" s="164"/>
+      <c r="X32" s="164"/>
+      <c r="Y32" s="164"/>
+    </row>
+    <row r="33" spans="1:25">
+      <c r="A33" s="153">
         <v>27</v>
       </c>
-      <c r="B33" s="170" t="s">
+      <c r="B33" s="155" t="s">
         <v>124</v>
       </c>
-      <c r="C33" s="170" t="s">
+      <c r="C33" s="155" t="s">
         <v>123</v>
       </c>
-      <c r="D33" s="168">
+      <c r="D33" s="153">
         <v>30849483</v>
       </c>
-      <c r="E33" s="172"/>
-      <c r="F33" s="176"/>
-      <c r="G33" s="172"/>
-      <c r="H33" s="172">
+      <c r="E33" s="26">
+        <v>20241130214</v>
+      </c>
+      <c r="F33" s="157"/>
+      <c r="G33" s="160"/>
+      <c r="H33" s="157"/>
+      <c r="I33" s="157">
         <v>2</v>
       </c>
-      <c r="I33" s="172"/>
-      <c r="J33" s="172">
-        <v>1</v>
-      </c>
-      <c r="K33" s="172"/>
-      <c r="L33" s="172"/>
-      <c r="N33" s="172">
-        <v>1</v>
-      </c>
-      <c r="P33" s="172">
-        <v>1</v>
-      </c>
-      <c r="Q33" s="172"/>
-      <c r="R33" s="172"/>
-      <c r="S33" s="174">
+      <c r="J33" s="157"/>
+      <c r="K33" s="157">
+        <v>1</v>
+      </c>
+      <c r="L33" s="157"/>
+      <c r="M33" s="157"/>
+      <c r="O33" s="157">
+        <v>1</v>
+      </c>
+      <c r="Q33" s="157">
+        <v>1</v>
+      </c>
+      <c r="R33" s="157"/>
+      <c r="S33" s="157"/>
+      <c r="T33" s="159">
         <v>2</v>
       </c>
-      <c r="T33" s="174">
+      <c r="U33" s="159">
         <v>2</v>
       </c>
-      <c r="W33" s="174">
-        <v>1</v>
-      </c>
-      <c r="X33" s="174"/>
-    </row>
-    <row r="34" spans="1:24">
-      <c r="A34" s="168">
+      <c r="X33" s="159">
+        <v>1</v>
+      </c>
+      <c r="Y33" s="159"/>
+    </row>
+    <row r="34" spans="1:25">
+      <c r="A34" s="153">
         <v>28</v>
       </c>
-      <c r="B34" s="171" t="s">
+      <c r="B34" s="156" t="s">
         <v>128</v>
       </c>
-      <c r="C34" s="171" t="s">
+      <c r="C34" s="156" t="s">
         <v>127</v>
       </c>
-      <c r="D34" s="169">
+      <c r="D34" s="154">
         <v>31382931</v>
       </c>
-      <c r="E34" s="173">
-        <v>1</v>
-      </c>
-      <c r="F34" s="177">
+      <c r="E34" s="26">
+        <v>20251110444</v>
+      </c>
+      <c r="F34" s="158">
+        <v>1</v>
+      </c>
+      <c r="G34" s="161">
         <v>2</v>
       </c>
-      <c r="G34" s="178">
+      <c r="H34" s="162">
         <v>2</v>
       </c>
-      <c r="H34" s="173">
+      <c r="I34" s="158">
         <v>2</v>
       </c>
-      <c r="I34" s="173">
-        <v>1</v>
-      </c>
-      <c r="J34" s="178">
+      <c r="J34" s="158">
+        <v>1</v>
+      </c>
+      <c r="K34" s="162">
         <v>2</v>
       </c>
-      <c r="K34" s="178"/>
-      <c r="L34" s="173">
+      <c r="L34" s="162"/>
+      <c r="M34" s="158">
         <v>2</v>
       </c>
-      <c r="N34" s="173"/>
-      <c r="P34" s="173">
-        <v>1</v>
-      </c>
-      <c r="Q34" s="173">
+      <c r="O34" s="158"/>
+      <c r="Q34" s="158">
+        <v>1</v>
+      </c>
+      <c r="R34" s="158">
         <v>3</v>
       </c>
-      <c r="R34" s="173">
-        <v>1</v>
-      </c>
-      <c r="S34" s="180"/>
-      <c r="T34" s="180"/>
-      <c r="W34" s="180">
-        <v>1</v>
-      </c>
-      <c r="X34" s="180"/>
-    </row>
-    <row r="35" spans="1:24">
-      <c r="A35" s="169">
+      <c r="S34" s="158">
+        <v>1</v>
+      </c>
+      <c r="T34" s="164"/>
+      <c r="U34" s="164"/>
+      <c r="X34" s="164">
+        <v>1</v>
+      </c>
+      <c r="Y34" s="164"/>
+    </row>
+    <row r="35" spans="1:25">
+      <c r="A35" s="154">
         <v>29</v>
       </c>
-      <c r="B35" s="170" t="s">
+      <c r="B35" s="155" t="s">
         <v>132</v>
       </c>
-      <c r="C35" s="170" t="s">
+      <c r="C35" s="155" t="s">
         <v>131</v>
       </c>
-      <c r="D35" s="168">
+      <c r="D35" s="153">
         <v>32336250</v>
       </c>
-      <c r="E35" s="172"/>
-      <c r="F35" s="176"/>
-      <c r="G35" s="172"/>
-      <c r="H35" s="172"/>
-      <c r="I35" s="172"/>
-      <c r="J35" s="172"/>
-      <c r="K35" s="172"/>
-      <c r="L35" s="172"/>
-      <c r="N35" s="172"/>
-      <c r="P35" s="172"/>
-      <c r="Q35" s="172"/>
-      <c r="R35" s="172"/>
-      <c r="S35" s="174"/>
-      <c r="T35" s="174"/>
-      <c r="W35" s="174"/>
-      <c r="X35" s="174"/>
-    </row>
-    <row r="36" spans="1:24">
-      <c r="A36" s="168">
+      <c r="E35" s="26">
+        <v>20251110554</v>
+      </c>
+      <c r="F35" s="157"/>
+      <c r="G35" s="160"/>
+      <c r="H35" s="157"/>
+      <c r="I35" s="157"/>
+      <c r="J35" s="157"/>
+      <c r="K35" s="157"/>
+      <c r="L35" s="157"/>
+      <c r="M35" s="157"/>
+      <c r="O35" s="157"/>
+      <c r="Q35" s="157"/>
+      <c r="R35" s="157"/>
+      <c r="S35" s="157"/>
+      <c r="T35" s="159"/>
+      <c r="U35" s="159"/>
+      <c r="X35" s="159"/>
+      <c r="Y35" s="159"/>
+    </row>
+    <row r="36" spans="1:25">
+      <c r="A36" s="153">
         <v>30</v>
       </c>
-      <c r="B36" s="171" t="s">
+      <c r="B36" s="156" t="s">
         <v>108</v>
       </c>
-      <c r="C36" s="171" t="s">
+      <c r="C36" s="156" t="s">
         <v>135</v>
       </c>
-      <c r="D36" s="169">
+      <c r="D36" s="154">
         <v>32001498</v>
       </c>
-      <c r="E36" s="173"/>
-      <c r="F36" s="177"/>
-      <c r="G36" s="173"/>
-      <c r="H36" s="173">
+      <c r="E36" s="26">
+        <v>20251110262</v>
+      </c>
+      <c r="F36" s="158"/>
+      <c r="G36" s="161"/>
+      <c r="H36" s="158"/>
+      <c r="I36" s="158">
         <v>2</v>
       </c>
-      <c r="I36" s="173">
+      <c r="J36" s="158">
         <v>3</v>
       </c>
-      <c r="J36" s="179">
+      <c r="K36" s="163">
         <v>2</v>
       </c>
-      <c r="K36" s="179"/>
-      <c r="L36" s="179">
+      <c r="L36" s="163"/>
+      <c r="M36" s="163">
         <v>2</v>
       </c>
-      <c r="N36" s="179"/>
-      <c r="P36" s="179">
-        <v>1</v>
-      </c>
-      <c r="Q36" s="179">
-        <v>1</v>
-      </c>
-      <c r="R36" s="173"/>
-      <c r="S36" s="180"/>
-      <c r="T36" s="180">
+      <c r="O36" s="163"/>
+      <c r="Q36" s="163">
+        <v>1</v>
+      </c>
+      <c r="R36" s="163">
+        <v>1</v>
+      </c>
+      <c r="S36" s="158"/>
+      <c r="T36" s="164"/>
+      <c r="U36" s="164">
         <v>2</v>
       </c>
-      <c r="W36" s="180"/>
-      <c r="X36" s="180">
+      <c r="X36" s="164"/>
+      <c r="Y36" s="164">
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:24">
-      <c r="E37" s="175"/>
-      <c r="G37" s="175"/>
-      <c r="H37" s="175"/>
-      <c r="I37" s="175"/>
-      <c r="J37" s="175"/>
-      <c r="K37" s="175"/>
-      <c r="L37" s="175"/>
+    <row r="37" spans="1:25">
+      <c r="F37" s="1"/>
+      <c r="H37" s="1"/>
+      <c r="I37" s="1"/>
+      <c r="J37" s="1"/>
+      <c r="K37" s="1"/>
+      <c r="L37" s="1"/>
+      <c r="M37" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="16">
-    <mergeCell ref="AA5:AB5"/>
-    <mergeCell ref="Q5:R5"/>
-    <mergeCell ref="S5:T5"/>
-    <mergeCell ref="U5:V5"/>
-    <mergeCell ref="W5:X5"/>
-    <mergeCell ref="Y5:Z5"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="K5:L5"/>
-    <mergeCell ref="M5:N5"/>
-    <mergeCell ref="O5:P5"/>
+  <mergeCells count="17">
     <mergeCell ref="A5:A6"/>
     <mergeCell ref="B5:B6"/>
     <mergeCell ref="C5:C6"/>
     <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="N5:O5"/>
+    <mergeCell ref="P5:Q5"/>
+    <mergeCell ref="AB5:AC5"/>
+    <mergeCell ref="R5:S5"/>
+    <mergeCell ref="T5:U5"/>
+    <mergeCell ref="V5:W5"/>
+    <mergeCell ref="X5:Y5"/>
+    <mergeCell ref="Z5:AA5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -14924,7 +15129,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="15" customHeight="1"/>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="153" t="s">
+      <c r="A1" s="166" t="s">
         <v>2</v>
       </c>
       <c r="B1" s="13" t="s">
@@ -14942,12 +15147,12 @@
       <c r="F1" s="14" t="s">
         <v>141</v>
       </c>
-      <c r="G1" s="153" t="s">
+      <c r="G1" s="166" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="154"/>
+      <c r="A2" s="167"/>
       <c r="B2" s="15" t="s">
         <v>143</v>
       </c>
@@ -14963,7 +15168,7 @@
       <c r="F2" s="16" t="s">
         <v>143</v>
       </c>
-      <c r="G2" s="154"/>
+      <c r="G2" s="167"/>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="17" t="s">
@@ -16479,29 +16684,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
-      <c r="A1" s="155" t="s">
+      <c r="A1" s="168" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="157" t="s">
+      <c r="B1" s="170" t="s">
         <v>183</v>
       </c>
-      <c r="C1" s="158"/>
-      <c r="D1" s="158"/>
-      <c r="E1" s="158"/>
-      <c r="F1" s="158"/>
-      <c r="G1" s="158"/>
-      <c r="H1" s="158"/>
-      <c r="I1" s="159"/>
-      <c r="J1" s="160" t="s">
+      <c r="C1" s="171"/>
+      <c r="D1" s="171"/>
+      <c r="E1" s="171"/>
+      <c r="F1" s="171"/>
+      <c r="G1" s="171"/>
+      <c r="H1" s="171"/>
+      <c r="I1" s="172"/>
+      <c r="J1" s="173" t="s">
         <v>141</v>
       </c>
-      <c r="K1" s="161"/>
-      <c r="L1" s="162" t="s">
+      <c r="K1" s="174"/>
+      <c r="L1" s="175" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="2" spans="1:12">
-      <c r="A2" s="156"/>
+      <c r="A2" s="169"/>
       <c r="B2" s="40" t="s">
         <v>184</v>
       </c>
@@ -16532,7 +16737,7 @@
       <c r="K2" s="41" t="s">
         <v>193</v>
       </c>
-      <c r="L2" s="163"/>
+      <c r="L2" s="176"/>
     </row>
     <row r="3" spans="1:12">
       <c r="A3" s="42" t="s">
@@ -18041,41 +18246,41 @@
       <c r="C1" s="38"/>
       <c r="D1" s="38"/>
       <c r="E1" s="38"/>
-      <c r="F1" s="164" t="s">
+      <c r="F1" s="177" t="s">
         <v>206</v>
       </c>
       <c r="G1" s="165"/>
       <c r="H1" s="165"/>
-      <c r="I1" s="166"/>
+      <c r="I1" s="178"/>
       <c r="J1" s="38"/>
-      <c r="K1" s="164" t="s">
+      <c r="K1" s="177" t="s">
         <v>207</v>
       </c>
       <c r="L1" s="165"/>
-      <c r="M1" s="166"/>
-      <c r="N1" s="167" t="s">
+      <c r="M1" s="178"/>
+      <c r="N1" s="179" t="s">
         <v>208</v>
       </c>
       <c r="O1" s="165"/>
       <c r="P1" s="165"/>
-      <c r="Q1" s="164" t="s">
+      <c r="Q1" s="177" t="s">
         <v>209</v>
       </c>
       <c r="R1" s="165"/>
-      <c r="S1" s="166"/>
-      <c r="T1" s="167" t="s">
+      <c r="S1" s="178"/>
+      <c r="T1" s="179" t="s">
         <v>210</v>
       </c>
       <c r="U1" s="165"/>
       <c r="V1" s="165"/>
-      <c r="W1" s="164" t="s">
+      <c r="W1" s="177" t="s">
         <v>211</v>
       </c>
-      <c r="X1" s="166"/>
-      <c r="Y1" s="167" t="s">
+      <c r="X1" s="178"/>
+      <c r="Y1" s="179" t="s">
         <v>212</v>
       </c>
-      <c r="Z1" s="166"/>
+      <c r="Z1" s="178"/>
       <c r="AA1" s="38"/>
     </row>
     <row r="2" spans="1:27">

</xml_diff>

<commit_message>
Primeros csv en downstream
</commit_message>
<xml_diff>
--- a/Datos Tesis Upstream/Algoritmos y Programacion/2425-2/Partic.Alg 2425-2 Secc. 1.xlsx
+++ b/Datos Tesis Upstream/Algoritmos y Programacion/2425-2/Partic.Alg 2425-2 Secc. 1.xlsx
@@ -24,6 +24,7 @@
     <sheet name="Tareas" sheetId="9" r:id="rId9"/>
     <sheet name="Xtra" sheetId="10" r:id="rId10"/>
     <sheet name="Estandar" sheetId="11" r:id="rId11"/>
+    <sheet name="Cronograma" sheetId="12" r:id="rId19"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -14052,102 +14053,102 @@
       <c r="Y13" s="159"/>
     </row>
     <row r="14" spans="1:29">
-      <c r="A14" s="154">
+      <c r="A14" s="153">
         <v>8</v>
       </c>
-      <c r="B14" s="156" t="s">
+      <c r="B14" s="155" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14" s="155" t="s">
+        <v>51</v>
+      </c>
+      <c r="D14" s="153">
+        <v>32042714</v>
+      </c>
+      <c r="E14" s="26">
+        <v>20251110345</v>
+      </c>
+      <c r="F14" s="157"/>
+      <c r="G14" s="160"/>
+      <c r="H14" s="157"/>
+      <c r="I14" s="157"/>
+      <c r="J14" s="157">
+        <v>2</v>
+      </c>
+      <c r="K14" s="157"/>
+      <c r="L14" s="157">
+        <v>2</v>
+      </c>
+      <c r="M14" s="157">
+        <v>1</v>
+      </c>
+      <c r="O14" s="157">
+        <v>1</v>
+      </c>
+      <c r="Q14" s="157">
+        <v>1</v>
+      </c>
+      <c r="R14" s="157">
+        <v>1</v>
+      </c>
+      <c r="S14" s="157">
+        <v>1</v>
+      </c>
+      <c r="T14" s="157">
+        <v>3</v>
+      </c>
+      <c r="U14" s="159">
+        <v>3</v>
+      </c>
+      <c r="X14" s="159">
+        <v>1</v>
+      </c>
+      <c r="Y14" s="159"/>
+    </row>
+    <row r="15" spans="1:29">
+      <c r="A15" s="154">
+        <v>9</v>
+      </c>
+      <c r="B15" s="156" t="s">
         <v>48</v>
       </c>
-      <c r="C14" s="156" t="s">
+      <c r="C15" s="156" t="s">
         <v>47</v>
       </c>
-      <c r="D14" s="154">
+      <c r="D15" s="154">
         <v>31979046</v>
       </c>
-      <c r="E14" s="26">
+      <c r="E15" s="26">
         <v>20241130202</v>
       </c>
-      <c r="F14" s="158"/>
-      <c r="G14" s="161">
+      <c r="F15" s="158"/>
+      <c r="G15" s="161">
         <v>2</v>
       </c>
-      <c r="H14" s="158"/>
-      <c r="I14" s="158"/>
-      <c r="J14" s="158"/>
-      <c r="K14" s="158"/>
-      <c r="L14" s="158"/>
-      <c r="M14" s="158">
+      <c r="H15" s="158"/>
+      <c r="I15" s="158"/>
+      <c r="J15" s="158"/>
+      <c r="K15" s="158"/>
+      <c r="L15" s="158"/>
+      <c r="M15" s="158">
         <v>2</v>
       </c>
-      <c r="O14" s="158"/>
-      <c r="Q14" s="158"/>
-      <c r="R14" s="158"/>
-      <c r="S14" s="158">
-        <v>1</v>
-      </c>
-      <c r="T14" s="164">
-        <v>1</v>
-      </c>
-      <c r="U14" s="164"/>
-      <c r="X14" s="164">
-        <v>1</v>
-      </c>
-      <c r="Y14" s="164">
+      <c r="O15" s="158"/>
+      <c r="Q15" s="158"/>
+      <c r="R15" s="158"/>
+      <c r="S15" s="158">
+        <v>1</v>
+      </c>
+      <c r="T15" s="164">
+        <v>1</v>
+      </c>
+      <c r="U15" s="164"/>
+      <c r="X15" s="164">
+        <v>1</v>
+      </c>
+      <c r="Y15" s="164">
         <v>2</v>
       </c>
-    </row>
-    <row r="15" spans="1:29">
-      <c r="A15" s="153">
-        <v>9</v>
-      </c>
-      <c r="B15" s="155" t="s">
-        <v>52</v>
-      </c>
-      <c r="C15" s="155" t="s">
-        <v>51</v>
-      </c>
-      <c r="D15" s="153">
-        <v>32042714</v>
-      </c>
-      <c r="E15" s="26">
-        <v>20251110345</v>
-      </c>
-      <c r="F15" s="157"/>
-      <c r="G15" s="160"/>
-      <c r="H15" s="157"/>
-      <c r="I15" s="157"/>
-      <c r="J15" s="157">
-        <v>2</v>
-      </c>
-      <c r="K15" s="157"/>
-      <c r="L15" s="157">
-        <v>2</v>
-      </c>
-      <c r="M15" s="157">
-        <v>1</v>
-      </c>
-      <c r="O15" s="157">
-        <v>1</v>
-      </c>
-      <c r="Q15" s="157">
-        <v>1</v>
-      </c>
-      <c r="R15" s="157">
-        <v>1</v>
-      </c>
-      <c r="S15" s="157">
-        <v>1</v>
-      </c>
-      <c r="T15" s="157">
-        <v>3</v>
-      </c>
-      <c r="U15" s="159">
-        <v>3</v>
-      </c>
-      <c r="X15" s="159">
-        <v>1</v>
-      </c>
-      <c r="Y15" s="159"/>
     </row>
     <row r="16" spans="1:29">
       <c r="A16" s="153">
@@ -14592,143 +14593,143 @@
       <c r="Y25" s="159"/>
     </row>
     <row r="26" spans="1:25">
-      <c r="A26" s="154">
+      <c r="A26" s="153">
         <v>20</v>
       </c>
       <c r="B26" s="156" t="s">
+        <v>104</v>
+      </c>
+      <c r="C26" s="156" t="s">
+        <v>103</v>
+      </c>
+      <c r="D26" s="154">
+        <v>32511604</v>
+      </c>
+      <c r="E26" s="26">
+        <v>20251110113</v>
+      </c>
+      <c r="F26" s="158">
+        <v>2</v>
+      </c>
+      <c r="G26" s="161">
+        <v>2</v>
+      </c>
+      <c r="H26" s="158">
+        <v>1</v>
+      </c>
+      <c r="I26" s="158">
+        <v>1</v>
+      </c>
+      <c r="J26" s="158">
+        <v>1</v>
+      </c>
+      <c r="K26" s="158">
+        <v>1</v>
+      </c>
+      <c r="L26" s="158">
+        <v>3</v>
+      </c>
+      <c r="M26" s="158"/>
+      <c r="O26" s="158">
+        <v>1</v>
+      </c>
+      <c r="Q26" s="158">
+        <v>2</v>
+      </c>
+      <c r="R26" s="158">
+        <v>3</v>
+      </c>
+      <c r="S26" s="158">
+        <v>3</v>
+      </c>
+      <c r="T26" s="164">
+        <v>1</v>
+      </c>
+      <c r="U26" s="164">
+        <v>1</v>
+      </c>
+      <c r="X26" s="164">
+        <v>1</v>
+      </c>
+      <c r="Y26" s="164">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:25">
+      <c r="A27" s="154">
+        <v>21</v>
+      </c>
+      <c r="B27" s="156" t="s">
         <v>96</v>
       </c>
-      <c r="C26" s="156" t="s">
+      <c r="C27" s="156" t="s">
         <v>95</v>
       </c>
-      <c r="D26" s="154">
+      <c r="D27" s="154">
         <v>31935917</v>
       </c>
-      <c r="E26" s="26">
+      <c r="E27" s="26">
         <v>20241130163</v>
       </c>
-      <c r="F26" s="158"/>
-      <c r="G26" s="161">
-        <v>1</v>
-      </c>
-      <c r="H26" s="162">
+      <c r="F27" s="158"/>
+      <c r="G27" s="161">
+        <v>1</v>
+      </c>
+      <c r="H27" s="162">
         <v>2</v>
       </c>
-      <c r="I26" s="158"/>
-      <c r="J26" s="158">
-        <v>1</v>
-      </c>
-      <c r="K26" s="158"/>
-      <c r="L26" s="158"/>
-      <c r="M26" s="158"/>
-      <c r="O26" s="158"/>
-      <c r="Q26" s="158"/>
-      <c r="R26" s="158"/>
-      <c r="S26" s="158"/>
-      <c r="T26" s="164"/>
-      <c r="U26" s="164"/>
-      <c r="X26" s="164"/>
-      <c r="Y26" s="164"/>
-    </row>
-    <row r="27" spans="1:25">
-      <c r="A27" s="153">
-        <v>21</v>
-      </c>
-      <c r="B27" s="155" t="s">
-        <v>100</v>
-      </c>
-      <c r="C27" s="155" t="s">
-        <v>99</v>
-      </c>
-      <c r="D27" s="153">
-        <v>31745168</v>
-      </c>
-      <c r="E27" s="26">
-        <v>20251110259</v>
-      </c>
-      <c r="F27" s="157"/>
-      <c r="G27" s="160"/>
-      <c r="H27" s="157"/>
-      <c r="I27" s="157"/>
-      <c r="J27" s="157"/>
-      <c r="K27" s="157"/>
-      <c r="L27" s="157"/>
-      <c r="M27" s="157"/>
-      <c r="O27" s="157">
-        <v>1</v>
-      </c>
-      <c r="Q27" s="157">
-        <v>1</v>
-      </c>
-      <c r="R27" s="157"/>
-      <c r="S27" s="157"/>
-      <c r="T27" s="159"/>
-      <c r="U27" s="159"/>
-      <c r="X27" s="159"/>
-      <c r="Y27" s="159"/>
+      <c r="I27" s="158"/>
+      <c r="J27" s="158">
+        <v>1</v>
+      </c>
+      <c r="K27" s="158"/>
+      <c r="L27" s="158"/>
+      <c r="M27" s="158"/>
+      <c r="O27" s="158"/>
+      <c r="Q27" s="158"/>
+      <c r="R27" s="158"/>
+      <c r="S27" s="158"/>
+      <c r="T27" s="164"/>
+      <c r="U27" s="164"/>
+      <c r="X27" s="164"/>
+      <c r="Y27" s="164"/>
     </row>
     <row r="28" spans="1:25">
       <c r="A28" s="153">
         <v>22</v>
       </c>
-      <c r="B28" s="156" t="s">
-        <v>104</v>
-      </c>
-      <c r="C28" s="156" t="s">
-        <v>103</v>
-      </c>
-      <c r="D28" s="154">
-        <v>32511604</v>
+      <c r="B28" s="155" t="s">
+        <v>100</v>
+      </c>
+      <c r="C28" s="155" t="s">
+        <v>99</v>
+      </c>
+      <c r="D28" s="153">
+        <v>31745168</v>
       </c>
       <c r="E28" s="26">
-        <v>20251110113</v>
-      </c>
-      <c r="F28" s="158">
-        <v>2</v>
-      </c>
-      <c r="G28" s="161">
-        <v>2</v>
-      </c>
-      <c r="H28" s="158">
-        <v>1</v>
-      </c>
-      <c r="I28" s="158">
-        <v>1</v>
-      </c>
-      <c r="J28" s="158">
-        <v>1</v>
-      </c>
-      <c r="K28" s="158">
-        <v>1</v>
-      </c>
-      <c r="L28" s="158">
-        <v>3</v>
-      </c>
-      <c r="M28" s="158"/>
-      <c r="O28" s="158">
-        <v>1</v>
-      </c>
-      <c r="Q28" s="158">
-        <v>2</v>
-      </c>
-      <c r="R28" s="158">
-        <v>3</v>
-      </c>
-      <c r="S28" s="158">
-        <v>3</v>
-      </c>
-      <c r="T28" s="164">
-        <v>1</v>
-      </c>
-      <c r="U28" s="164">
-        <v>1</v>
-      </c>
-      <c r="X28" s="164">
-        <v>1</v>
-      </c>
-      <c r="Y28" s="164">
-        <v>1</v>
-      </c>
+        <v>20251110259</v>
+      </c>
+      <c r="F28" s="157"/>
+      <c r="G28" s="160"/>
+      <c r="H28" s="157"/>
+      <c r="I28" s="157"/>
+      <c r="J28" s="157"/>
+      <c r="K28" s="157"/>
+      <c r="L28" s="157"/>
+      <c r="M28" s="157"/>
+      <c r="O28" s="157">
+        <v>1</v>
+      </c>
+      <c r="Q28" s="157">
+        <v>1</v>
+      </c>
+      <c r="R28" s="157"/>
+      <c r="S28" s="157"/>
+      <c r="T28" s="159"/>
+      <c r="U28" s="159"/>
+      <c r="X28" s="159"/>
+      <c r="Y28" s="159"/>
     </row>
     <row r="29" spans="1:25">
       <c r="A29" s="154">
@@ -15117,6 +15118,372 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="8" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">semana</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dia_sesion</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tema</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tipo_sesion</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">administrativa</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>2</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>3</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>3</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>4</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>4</v>
+      </c>
+      <c r="B9">
+        <v>2</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">repaso</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>5</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">evaluacion</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>5</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>6</v>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">evaluacion</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>6</v>
+      </c>
+      <c r="B13">
+        <v>2</v>
+      </c>
+      <c r="C13">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>7</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>7</v>
+      </c>
+      <c r="B15">
+        <v>2</v>
+      </c>
+      <c r="C15">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>8</v>
+      </c>
+      <c r="B16">
+        <v>1</v>
+      </c>
+      <c r="C16">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>8</v>
+      </c>
+      <c r="B17">
+        <v>2</v>
+      </c>
+      <c r="C17">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>9</v>
+      </c>
+      <c r="B18">
+        <v>1</v>
+      </c>
+      <c r="C18">
+        <v>0</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sin_clase</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>9</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19">
+        <v>0</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">evaluacion</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <v>10</v>
+      </c>
+      <c r="B20">
+        <v>1</v>
+      </c>
+      <c r="C20">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <v>10</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21">
+        <v>0</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">repaso</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <v>11</v>
+      </c>
+      <c r="B22">
+        <v>1</v>
+      </c>
+      <c r="C22">
+        <v>0</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">evaluacion</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23">
+        <v>11</v>
+      </c>
+      <c r="B23">
+        <v>2</v>
+      </c>
+      <c r="C23">
+        <v>0</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">evaluacion</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <v>12</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24">
+        <v>0</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">administrativa</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25">
+        <v>12</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25">
+        <v>0</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">administrativa</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nota:</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tema = código del catálogo de la asignatura. Si la sesión no cubre contenido nuevo: tema = 0 y tipo_sesion indica la causa (evaluacion, repaso, sin_clase, administrativa). Si tema &gt; 0 la sesión es de contenido y tipo_sesion queda vacío.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
 </worksheet>
 </file>
 

</xml_diff>